<commit_message>
vault backup: 2026-03-28 11:04:43
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -1,130 +1,151 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52C59588-A6F6-4179-BBDE-8C5FC013AB20}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
+    <sheet name="Hoja5" sheetId="5" r:id="rId5"/>
+    <sheet name="Hoja6" sheetId="6" r:id="rId6"/>
+    <sheet name="Hoja7" sheetId="7" r:id="rId7"/>
+    <sheet name="Hoja8" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
+    <definedName name="solver_adj" localSheetId="0" hidden="1">Hoja1!$B$5:$C$5</definedName>
+    <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
+    <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
+    <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
+    <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
+    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
+    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
+    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
+    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
+    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
+    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
+    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
+    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rel6" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
+    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
+    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
+    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
+    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
+    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
+    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
+    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
+    <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
-    <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_adj" localSheetId="0" hidden="1">Hoja1!$B$5:$C$5</definedName>
-    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
-    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
-    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
-    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
-    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
-    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
-    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
-    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
-    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
-    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
-    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
-    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
-    <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
-    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
-    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
-    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
-    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
-    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
-    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
-    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
-    <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
-    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
-    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
-    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
-    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
-    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
-    <definedName name="solver_rel5" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
-    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
-    <definedName name="solver_rel6" localSheetId="3" hidden="1">2</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
   <si>
-    <t xml:space="preserve">Tipo de carne</t>
+    <t>Tipo de carne</t>
   </si>
   <si>
     <t>R</t>
@@ -205,10 +226,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -224,18 +245,18 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -253,291 +274,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -728,17 +466,19 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.00390625"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="14.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -747,7 +487,7 @@
         <v>716.66666666666742</v>
       </c>
     </row>
-    <row r="4" ht="14.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -758,7 +498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" ht="14.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -769,7 +509,7 @@
         <v>0.41666666666666702</v>
       </c>
     </row>
-    <row r="6" ht="14.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -780,7 +520,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="8" ht="14.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -788,15 +528,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" ht="14.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C9">
-        <v>0.32000000000000001</v>
+        <v>0.32</v>
       </c>
       <c r="D9">
         <f>B5*B9+C5*C9</f>
@@ -809,7 +549,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" ht="14.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
@@ -828,21 +568,20 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A2:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="12.7109375"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -851,7 +590,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -862,7 +601,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>20</v>
       </c>
@@ -870,7 +609,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -881,12 +620,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>2</v>
       </c>
@@ -904,7 +643,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
@@ -922,7 +661,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>1</v>
       </c>
@@ -938,18 +677,17 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -958,7 +696,7 @@
         <v>7.2727272727272751</v>
       </c>
     </row>
-    <row r="2" ht="14.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -981,7 +719,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" ht="14.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>0.90909090909090895</v>
       </c>
@@ -1001,7 +739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" ht="14.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>2</v>
       </c>
@@ -1021,12 +759,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="14.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" ht="14.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>20</v>
       </c>
@@ -1056,7 +794,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" ht="14.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>50</v>
       </c>
@@ -1086,7 +824,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" ht="14.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>4</v>
       </c>
@@ -1117,18 +855,17 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" ht="14.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1137,7 +874,7 @@
         <v>1250000</v>
       </c>
     </row>
-    <row r="2" ht="14.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1154,7 +891,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" ht="14.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>50.000000000000014</v>
       </c>
@@ -1168,7 +905,7 @@
         <v>10.000000000000004</v>
       </c>
     </row>
-    <row r="4" ht="14.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>6000</v>
       </c>
@@ -1182,12 +919,12 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="5" ht="14.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" ht="14.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>3</v>
       </c>
@@ -1211,7 +948,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="7" ht="14.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1235,7 +972,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" ht="14.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>2</v>
       </c>
@@ -1259,7 +996,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" ht="14.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E9">
         <v>1</v>
       </c>
@@ -1274,7 +1011,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" ht="14.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
@@ -1289,7 +1026,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" ht="14.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>1</v>
       </c>
@@ -1311,9 +1048,43 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988A02B7-B628-469A-96AE-572BC7342D70}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB7A058-7B66-4047-8F0A-EA5D43949925}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FEE52C-5C57-4D5C-BDBD-8B72D286EB32}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F599C5-62BA-4458-915A-A99270222596}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-03-28 11:14:48
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52C59588-A6F6-4179-BBDE-8C5FC013AB20}"/>
+  <xr:revisionPtr revIDLastSave="316" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82991B88-4FE8-4CEF-894A-7F5647DB0AB0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10995" yWindow="0" windowWidth="17910" windowHeight="15585" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -27,63 +27,98 @@
     <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
     <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
     <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
+    <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
+    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
     <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
     <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
     <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
     <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
     <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
     <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
     <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
     <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
     <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
     <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
     <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
     <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
+    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
+    <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
     <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rel6" localSheetId="3" hidden="1">2</definedName>
@@ -91,36 +126,56 @@
     <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
     <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
     <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
     <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
     <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
     <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
     <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
     <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
     <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
     <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
     <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
     <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
+    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -140,7 +195,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="30">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
@@ -221,17 +276,33 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;= </t>
+  </si>
+  <si>
+    <t>Ganancias</t>
+  </si>
+  <si>
+    <t>Carne</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -255,8 +326,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1055,18 +1127,225 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988A02B7-B628-469A-96AE-572BC7342D70}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1">
+        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>11.428571428571429</v>
+      </c>
+      <c r="C3">
+        <v>5.7142857142857144</v>
+      </c>
+      <c r="D3">
+        <v>5.7142857142857144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>700</v>
+      </c>
+      <c r="C4">
+        <v>2100</v>
+      </c>
+      <c r="D4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <f>SUMPRODUCT(B3:D3,B6:D6)</f>
+        <v>40</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>-2</v>
+      </c>
+      <c r="E7">
+        <f>SUMPRODUCT(B3:C3,B7:C7)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>-1</v>
+      </c>
+      <c r="E8">
+        <f>SUMPRODUCT(C3:D3,C8:D8)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E7:E8" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB7A058-7B66-4047-8F0A-EA5D43949925}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1">
+        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
+        <v>1255.0000021999999</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>200.000001</v>
+      </c>
+      <c r="C3">
+        <v>800.000001</v>
+      </c>
+      <c r="D3">
+        <v>150.000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>0.3</v>
+      </c>
+      <c r="C4">
+        <v>1.4</v>
+      </c>
+      <c r="D4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <f>B3*B6</f>
+        <v>200.000001</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <f>C3*C7</f>
+        <v>800.000001</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <f>D3*D8</f>
+        <v>150.000001</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
vault backup: 2026-03-28 11:24:51
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="316" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82991B88-4FE8-4CEF-894A-7F5647DB0AB0}"/>
+  <xr:revisionPtr revIDLastSave="511" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0AB4A65-A90C-41C2-8AD6-8AAF560B2E4D}"/>
   <bookViews>
-    <workbookView xWindow="10995" yWindow="0" windowWidth="17910" windowHeight="15585" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10995" yWindow="0" windowWidth="17910" windowHeight="15585" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,97 +29,122 @@
     <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
     <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
     <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja7!$B$3:$E$3</definedName>
     <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
     <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
     <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
     <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
     <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
     <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
     <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
     <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
     <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
     <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
     <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
     <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
     <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
     <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
     <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
     <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
     <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
+    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
     <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
     <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
     <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
     <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
     <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rel6" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
@@ -128,54 +153,68 @@
     <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
     <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
     <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
     <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
     <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
     <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
     <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
     <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
     <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
     <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
     <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
     <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
     <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
     <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
+    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
     <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
     <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
     <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -195,7 +234,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="39">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
@@ -285,6 +324,33 @@
   </si>
   <si>
     <t>L</t>
+  </si>
+  <si>
+    <t>Barriles</t>
+  </si>
+  <si>
+    <t>Restrricciones</t>
+  </si>
+  <si>
+    <t>NR</t>
+  </si>
+  <si>
+    <t>IR</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>Servicios</t>
+  </si>
+  <si>
+    <t>P</t>
   </si>
 </sst>
 </file>
@@ -1352,18 +1418,236 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FEE52C-5C57-4D5C-BDBD-8B72D286EB32}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1">
+        <f>SUMPRODUCT(B3:E3,B4:E4)</f>
+        <v>33907636547.368427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>7064090.9473684216</v>
+      </c>
+      <c r="E3">
+        <v>8476909.1368421055</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>4000</v>
+      </c>
+      <c r="C4">
+        <v>-3000</v>
+      </c>
+      <c r="D4">
+        <v>6000</v>
+      </c>
+      <c r="E4">
+        <v>-1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <f>SUMPRODUCT(B3:C3,B6:C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>-5</v>
+      </c>
+      <c r="F7">
+        <f>SUMPRODUCT(D3:E3,D7:E7)</f>
+        <v>7.4505805969238281E-9</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>-8</v>
+      </c>
+      <c r="F8">
+        <f>SUMPRODUCT(B3:C3,B8:C8)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>-8</v>
+      </c>
+      <c r="F9">
+        <f>SUMPRODUCT(D3:E3,D9:E9)</f>
+        <v>-53687091.200000003</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F599C5-62BA-4458-915A-A99270222596}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>100000</v>
+      </c>
+      <c r="C4">
+        <v>18000</v>
+      </c>
+      <c r="D4">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>20000</v>
+      </c>
+      <c r="C6">
+        <v>3000</v>
+      </c>
+      <c r="D6">
+        <v>6000</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="1">
+        <v>18500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-03-28 11:34:57
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="511" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0AB4A65-A90C-41C2-8AD6-8AAF560B2E4D}"/>
+  <xr:revisionPtr revIDLastSave="686" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01765DC9-F5E5-49E3-B697-3889E3AB8DAD}"/>
   <bookViews>
     <workbookView xWindow="10995" yWindow="0" windowWidth="17910" windowHeight="15585" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,10 +30,13 @@
     <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
     <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
     <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja7!$B$3:$E$3</definedName>
+    <definedName name="solver_adj" localSheetId="7" hidden="1">Hoja8!$B$3:$D$3</definedName>
     <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
@@ -41,12 +44,14 @@
     <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
@@ -54,6 +59,7 @@
     <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
     <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
     <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
@@ -61,6 +67,7 @@
     <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
     <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
     <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="7" hidden="1">Hoja8!$E$10</definedName>
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
     <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
     <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
@@ -68,24 +75,33 @@
     <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
     <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
     <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="7" hidden="1">Hoja8!$E$11</definedName>
     <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
     <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
     <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
     <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
     <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
     <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="7" hidden="1">Hoja8!$E$6</definedName>
     <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
     <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
+    <definedName name="solver_lhs4" localSheetId="7" hidden="1">Hoja8!$E$7</definedName>
     <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
+    <definedName name="solver_lhs5" localSheetId="7" hidden="1">Hoja8!$E$8</definedName>
     <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
+    <definedName name="solver_lhs6" localSheetId="7" hidden="1">Hoja8!$E$9</definedName>
     <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
@@ -93,8 +109,10 @@
     <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
@@ -102,12 +120,14 @@
     <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
+    <definedName name="solver_num" localSheetId="7" hidden="1">6</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
     <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
@@ -115,14 +135,17 @@
     <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="7" hidden="1">Hoja8!$B$1</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
@@ -130,6 +153,7 @@
     <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
@@ -137,16 +161,21 @@
     <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="7" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rel5" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rel6" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
     <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
     <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
@@ -154,6 +183,7 @@
     <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
     <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
     <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="7" hidden="1">Hoja8!$G$10</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
     <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
     <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
@@ -161,30 +191,40 @@
     <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
     <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
     <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="7" hidden="1">Hoja8!$G$11</definedName>
     <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
     <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
     <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
     <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
     <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
     <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="7" hidden="1">Hoja8!$G$6</definedName>
     <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
     <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
+    <definedName name="solver_rhs4" localSheetId="7" hidden="1">Hoja8!$G$7</definedName>
     <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
+    <definedName name="solver_rhs5" localSheetId="7" hidden="1">Hoja8!$G$8</definedName>
     <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
+    <definedName name="solver_rhs6" localSheetId="7" hidden="1">Hoja8!$G$9</definedName>
     <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
@@ -192,8 +232,10 @@
     <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
@@ -201,6 +243,7 @@
     <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
@@ -208,6 +251,7 @@
     <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
@@ -215,6 +259,7 @@
     <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="7" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -234,7 +279,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="39">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
@@ -357,7 +402,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -365,6 +410,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -392,9 +445,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1559,13 +1613,17 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F599C5-62BA-4458-915A-A99270222596}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="B1" s="2">
+        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
+        <v>114999.99974829119</v>
+      </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1581,6 +1639,17 @@
         <v>38</v>
       </c>
     </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>0.25000000755126428</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>2.2499999748291191</v>
+      </c>
+    </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>100000</v>
@@ -1607,6 +1676,10 @@
       <c r="D6">
         <v>6000</v>
       </c>
+      <c r="E6">
+        <f>SUMPRODUCT(B3:D3,B6:D6)</f>
+        <v>18500</v>
+      </c>
       <c r="F6" s="1" t="s">
         <v>9</v>
       </c>
@@ -1618,6 +1691,10 @@
       <c r="B7">
         <v>1</v>
       </c>
+      <c r="E7">
+        <f>B3*B7</f>
+        <v>0.25000000755126428</v>
+      </c>
       <c r="F7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1629,6 +1706,10 @@
       <c r="C8">
         <v>1</v>
       </c>
+      <c r="E8">
+        <f>C3*C8</f>
+        <v>0</v>
+      </c>
       <c r="F8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1640,11 +1721,57 @@
       <c r="D9">
         <v>1</v>
       </c>
+      <c r="E9">
+        <f>D3*D9</f>
+        <v>2.2499999748291191</v>
+      </c>
       <c r="F9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="G9">
         <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>-0.5</v>
+      </c>
+      <c r="C10">
+        <v>0.5</v>
+      </c>
+      <c r="D10">
+        <v>-0.5</v>
+      </c>
+      <c r="E10">
+        <f>SUMPRODUCT(B3:D3,B10:D10)</f>
+        <v>-1.2499999911901916</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>0.9</v>
+      </c>
+      <c r="C11">
+        <v>-0.1</v>
+      </c>
+      <c r="D11">
+        <v>-0.1</v>
+      </c>
+      <c r="E11">
+        <f>SUMPRODUCT(B3:D3,B11:D11)</f>
+        <v>9.3132259404438145E-9</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-04-02 12:19:39
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -1,290 +1,273 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="686" documentId="11_89FCA63F55AA6E97C9C88A334FFCC6A5FCACE4B7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01765DC9-F5E5-49E3-B697-3889E3AB8DAD}"/>
   <bookViews>
-    <workbookView xWindow="10995" yWindow="0" windowWidth="17910" windowHeight="15585" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
-    <sheet name="Hoja5" sheetId="5" r:id="rId5"/>
-    <sheet name="Hoja6" sheetId="6" r:id="rId6"/>
-    <sheet name="Hoja7" sheetId="7" r:id="rId7"/>
-    <sheet name="Hoja8" sheetId="8" r:id="rId8"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Hoja4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Hoja5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hoja6" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Hoja7" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Hoja8" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">Hoja1!$B$5:$C$5</definedName>
+    <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
+    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
+    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
+    <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
+    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
+    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
+    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
+    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
+    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
+    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
+    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
+    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
+    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
+    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
+    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
+    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
+    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
+    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
+    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
+    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
+    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
+    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
+    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
+    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
+    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
+    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
+    <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="3" hidden="1">3</definedName>
+    <definedName name="solver_rel6" localSheetId="3" hidden="1">3</definedName>
+    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
+    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
+    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
+    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
+    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
+    <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
+    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
+    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
+    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
+    <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
+    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
+    <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
+    <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
+    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
+    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
+    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
+    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
+    <definedName name="solver_pre" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
+    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
+    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_scl" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
+    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja7!$B$3:$E$3</definedName>
+    <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
+    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
+    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
+    <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
+    <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
+    <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
+    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
+    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
+    <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
+    <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
     <definedName name="solver_adj" localSheetId="7" hidden="1">Hoja8!$B$3:$D$3</definedName>
-    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
-    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
-    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
-    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
     <definedName name="solver_lhs1" localSheetId="7" hidden="1">Hoja8!$E$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
     <definedName name="solver_lhs2" localSheetId="7" hidden="1">Hoja8!$E$11</definedName>
-    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
-    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
     <definedName name="solver_lhs3" localSheetId="7" hidden="1">Hoja8!$E$6</definedName>
-    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
-    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
     <definedName name="solver_lhs4" localSheetId="7" hidden="1">Hoja8!$E$7</definedName>
-    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
     <definedName name="solver_lhs5" localSheetId="7" hidden="1">Hoja8!$E$8</definedName>
-    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
     <definedName name="solver_lhs6" localSheetId="7" hidden="1">Hoja8!$E$9</definedName>
-    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
-    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
-    <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
     <definedName name="solver_num" localSheetId="7" hidden="1">6</definedName>
-    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
-    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
-    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="7" hidden="1">Hoja8!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
-    <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
-    <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_rel2" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="7" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel5" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rel5" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel6" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rel6" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
-    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
-    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
     <definedName name="solver_rhs1" localSheetId="7" hidden="1">Hoja8!$G$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
     <definedName name="solver_rhs2" localSheetId="7" hidden="1">Hoja8!$G$11</definedName>
-    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
-    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
     <definedName name="solver_rhs3" localSheetId="7" hidden="1">Hoja8!$G$6</definedName>
-    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
-    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
     <definedName name="solver_rhs4" localSheetId="7" hidden="1">Hoja8!$G$7</definedName>
-    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
     <definedName name="solver_rhs5" localSheetId="7" hidden="1">Hoja8!$G$8</definedName>
-    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
     <definedName name="solver_rhs6" localSheetId="7" hidden="1">Hoja8!$G$9</definedName>
-    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
-    <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
-    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
-    <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
-    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="7" hidden="1">3</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
   <si>
-    <t>Tipo de carne</t>
+    <t xml:space="preserve">Tipo de carne</t>
   </si>
   <si>
     <t>R</t>
@@ -374,19 +357,19 @@
     <t>Barriles</t>
   </si>
   <si>
+    <t>NR</t>
+  </si>
+  <si>
+    <t>IR</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
     <t>Restrricciones</t>
-  </si>
-  <si>
-    <t>NR</t>
-  </si>
-  <si>
-    <t>IR</t>
-  </si>
-  <si>
-    <t>NE</t>
-  </si>
-  <si>
-    <t>IE</t>
   </si>
   <si>
     <t>?</t>
@@ -401,27 +384,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <u/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -435,20 +410,21 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="4">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,8 +442,291 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -658,19 +917,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:F10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="15"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -679,7 +936,7 @@
         <v>716.66666666666742</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -690,7 +947,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -701,7 +958,7 @@
         <v>0.41666666666666702</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -712,7 +969,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -720,15 +977,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.2</v>
+        <v>0.20000000000000001</v>
       </c>
       <c r="C9">
-        <v>0.32</v>
+        <v>0.32000000000000001</v>
       </c>
       <c r="D9">
         <f>B5*B9+C5*C9</f>
@@ -741,7 +998,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="B10">
         <v>1</v>
       </c>
@@ -760,20 +1017,21 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="12.7109375"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -782,7 +1040,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -793,7 +1051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="B5">
         <v>20</v>
       </c>
@@ -801,7 +1059,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -812,12 +1070,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="B9">
         <v>2</v>
       </c>
@@ -835,7 +1093,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="B10">
         <v>1</v>
       </c>
@@ -853,7 +1111,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="B11">
         <v>1</v>
       </c>
@@ -869,17 +1127,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -888,7 +1147,7 @@
         <v>7.2727272727272751</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -911,7 +1170,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="B3">
         <v>0.90909090909090895</v>
       </c>
@@ -931,7 +1190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="B4">
         <v>2</v>
       </c>
@@ -951,12 +1210,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="B6">
         <v>20</v>
       </c>
@@ -986,7 +1245,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="B7">
         <v>50</v>
       </c>
@@ -1016,7 +1275,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="B8">
         <v>4</v>
       </c>
@@ -1047,17 +1306,18 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1066,7 +1326,7 @@
         <v>1250000</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1083,9 +1343,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="B3">
-        <v>50.000000000000014</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1094,10 +1354,10 @@
         <v>145</v>
       </c>
       <c r="E3">
-        <v>10.000000000000004</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>9.9999999999999982</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="B4">
         <v>6000</v>
       </c>
@@ -1111,12 +1371,12 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="B6">
         <v>3</v>
       </c>
@@ -1131,7 +1391,7 @@
       </c>
       <c r="F6">
         <f>SUMPRODUCT(B3:E3,B6:E6)</f>
-        <v>480.00000000000006</v>
+        <v>480</v>
       </c>
       <c r="G6" t="s">
         <v>26</v>
@@ -1140,7 +1400,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1164,7 +1424,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="B8">
         <v>2</v>
       </c>
@@ -1188,13 +1448,13 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9">
         <f>E3*E9</f>
-        <v>10.000000000000004</v>
+        <v>9.9999999999999982</v>
       </c>
       <c r="G9" t="s">
         <v>26</v>
@@ -1203,22 +1463,22 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="B10">
         <v>1</v>
       </c>
       <c r="F10">
         <f>B3*B10</f>
-        <v>50.000000000000014</v>
+        <v>50</v>
       </c>
       <c r="G10" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="H10">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="B11">
         <v>1</v>
       </c>
@@ -1233,24 +1493,25 @@
         <v>195</v>
       </c>
       <c r="G11" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="H11">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988A02B7-B628-469A-96AE-572BC7342D70}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1259,7 +1520,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1273,7 +1534,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="B3">
         <v>11.428571428571429</v>
       </c>
@@ -1284,7 +1545,7 @@
         <v>5.7142857142857144</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="B4">
         <v>700</v>
       </c>
@@ -1295,12 +1556,12 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="B6">
         <v>1</v>
       </c>
@@ -1314,14 +1575,14 @@
         <f>SUMPRODUCT(B3:D3,B6:D6)</f>
         <v>40</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G6" s="1">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1339,7 +1600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="C8">
         <v>1</v>
       </c>
@@ -1358,28 +1619,32 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="E7:E8" formulaRange="1"/>
-  </ignoredErrors>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FB7A058-7B66-4047-8F0A-EA5D43949925}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B1">
         <f>SUMPRODUCT(B3:D3,B4:D4)</f>
-        <v>1255.0000021999999</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+    </row>
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
@@ -1392,90 +1657,126 @@
       <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+    </row>
+    <row r="3">
+      <c r="A3"/>
       <c r="B3">
-        <v>200.000001</v>
+        <v>0</v>
       </c>
       <c r="C3">
-        <v>800.000001</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>150.000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+    </row>
+    <row r="4">
+      <c r="A4"/>
       <c r="B4">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
+    </row>
+    <row r="5">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+      <c r="G5"/>
+    </row>
+    <row r="6">
+      <c r="A6"/>
       <c r="B6">
-        <v>1</v>
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="C6"/>
+      <c r="D6">
+        <v>0.10000000000000001</v>
       </c>
       <c r="E6">
-        <f>B3*B6</f>
-        <v>200.000001</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>10</v>
+        <f>B3*B6+D3*D6</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="G6">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7">
+      <c r="A7"/>
+      <c r="B7">
+        <v>0.5</v>
+      </c>
       <c r="C7">
-        <v>1</v>
+        <v>0.5</v>
+      </c>
+      <c r="D7">
+        <v>0.40000000000000002</v>
       </c>
       <c r="E7">
-        <f>C3*C7</f>
-        <v>800.000001</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>10</v>
+        <f>SUMPRODUCT($B$3:$D$3,B7:D7)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="G7">
         <v>800</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8">
+      <c r="A8"/>
+      <c r="B8"/>
+      <c r="C8">
+        <v>0.20000000000000001</v>
+      </c>
       <c r="D8">
-        <v>1</v>
+        <v>0.29999999999999999</v>
       </c>
       <c r="E8">
-        <f>D3*D8</f>
-        <v>150.000001</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>10</v>
+        <f>SUMPRODUCT(C3:D3,C8:D8)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="G8">
         <v>150</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FEE52C-5C57-4D5C-BDBD-8B72D286EB32}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -1484,24 +1785,24 @@
         <v>33907636547.368427</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3">
       <c r="B3">
         <v>0</v>
       </c>
@@ -1515,7 +1816,7 @@
         <v>8476909.1368421055</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="B4">
         <v>4000</v>
       </c>
@@ -1529,12 +1830,12 @@
         <v>-1000</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="B6">
         <v>1</v>
       </c>
@@ -1552,7 +1853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="D7">
         <v>6</v>
       </c>
@@ -1561,7 +1862,7 @@
       </c>
       <c r="F7">
         <f>SUMPRODUCT(D3:E3,D7:E7)</f>
-        <v>7.4505805969238281E-9</v>
+        <v>7.4505805969238281e-09</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>9</v>
@@ -1570,7 +1871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="B8">
         <v>2</v>
       </c>
@@ -1588,7 +1889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="D9">
         <v>2</v>
       </c>
@@ -1607,25 +1908,27 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F599C5-62BA-4458-915A-A99270222596}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="2">
+      <c r="B1" s="3">
         <f>SUMPRODUCT(B3:D3,B4:D4)</f>
         <v>114999.99974829119</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
@@ -1639,7 +1942,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="B3">
         <v>0.25000000755126428</v>
       </c>
@@ -1650,7 +1953,7 @@
         <v>2.2499999748291191</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="B4">
         <v>100000</v>
       </c>
@@ -1661,12 +1964,12 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="B6">
         <v>20000</v>
       </c>
@@ -1687,7 +1990,7 @@
         <v>18500</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1702,7 +2005,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="C8">
         <v>1</v>
       </c>
@@ -1717,7 +2020,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="D9">
         <v>1</v>
       </c>
@@ -1732,7 +2035,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="B10">
         <v>-0.5</v>
       </c>
@@ -1753,19 +2056,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="B11">
-        <v>0.9</v>
+        <v>0.90000000000000002</v>
       </c>
       <c r="C11">
-        <v>-0.1</v>
+        <v>-0.10000000000000001</v>
       </c>
       <c r="D11">
-        <v>-0.1</v>
+        <v>-0.10000000000000001</v>
       </c>
       <c r="E11">
         <f>SUMPRODUCT(B3:D3,B11:D11)</f>
-        <v>9.3132259404438145E-9</v>
+        <v>9.3132259404438145e-09</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>23</v>
@@ -1775,6 +2078,9 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-02 12:28:59
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -1,273 +1,290 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="195" documentId="11_25ECF59304F7134D1C4F5E9C0BAFF804774F75A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{945858A0-6763-4ACD-AE07-CE3098277BCB}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Hoja5" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Hoja6" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Hoja7" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Hoja8" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
+    <sheet name="Hoja5" sheetId="5" r:id="rId5"/>
+    <sheet name="Hoja6" sheetId="6" r:id="rId6"/>
+    <sheet name="Hoja7" sheetId="7" r:id="rId7"/>
+    <sheet name="Hoja8" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">Hoja1!$B$5:$C$5</definedName>
+    <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
+    <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
+    <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
+    <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja7!$B$3:$E$3</definedName>
+    <definedName name="solver_adj" localSheetId="7" hidden="1">Hoja8!$B$3:$D$3</definedName>
+    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="7" hidden="1">Hoja8!$E$10</definedName>
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="7" hidden="1">Hoja8!$E$11</definedName>
+    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
+    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="7" hidden="1">Hoja8!$E$6</definedName>
+    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
+    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
+    <definedName name="solver_lhs4" localSheetId="7" hidden="1">Hoja8!$E$7</definedName>
+    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
+    <definedName name="solver_lhs5" localSheetId="7" hidden="1">Hoja8!$E$8</definedName>
+    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
+    <definedName name="solver_lhs6" localSheetId="7" hidden="1">Hoja8!$E$9</definedName>
+    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
+    <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
+    <definedName name="solver_num" localSheetId="7" hidden="1">6</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
+    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
+    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="7" hidden="1">Hoja8!$B$1</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="5" hidden="1">0.0000001</definedName>
+    <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rel2" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="7" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="3" hidden="1">3</definedName>
+    <definedName name="solver_rel5" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_rel6" localSheetId="3" hidden="1">3</definedName>
+    <definedName name="solver_rel6" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
+    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
+    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="7" hidden="1">Hoja8!$G$10</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="7" hidden="1">Hoja8!$G$11</definedName>
+    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
+    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="7" hidden="1">Hoja8!$G$6</definedName>
+    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
+    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
+    <definedName name="solver_rhs4" localSheetId="7" hidden="1">Hoja8!$G$7</definedName>
+    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
+    <definedName name="solver_rhs5" localSheetId="7" hidden="1">Hoja8!$G$8</definedName>
+    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
+    <definedName name="solver_rhs6" localSheetId="7" hidden="1">Hoja8!$G$9</definedName>
+    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="7" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
-    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
-    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
-    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
-    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
-    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
-    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
-    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
-    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
-    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
-    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
-    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
-    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
-    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
-    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
-    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
-    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
-    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
-    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
-    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
-    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
-    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
-    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
-    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel5" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_rel6" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
-    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
-    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
-    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
-    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
-    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
-    <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
-    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
-    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
-    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
-    <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
-    <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
-    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
-    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
-    <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
-    <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
-    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
-    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
-    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
-    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
-    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
-    <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="5" hidden="1">0</definedName>
-    <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
-    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
-    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
-    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
-    <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
-    <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja7!$B$3:$E$3</definedName>
-    <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
-    <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
-    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
-    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
-    <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
-    <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
-    <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
-    <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
-    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
-    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
-    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
-    <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
-    <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
-    <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
-    <definedName name="solver_adj" localSheetId="7" hidden="1">Hoja8!$B$3:$D$3</definedName>
-    <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
-    <definedName name="solver_drv" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="7" hidden="1">Hoja8!$E$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="7" hidden="1">Hoja8!$E$11</definedName>
-    <definedName name="solver_lhs3" localSheetId="7" hidden="1">Hoja8!$E$6</definedName>
-    <definedName name="solver_lhs4" localSheetId="7" hidden="1">Hoja8!$E$7</definedName>
-    <definedName name="solver_lhs5" localSheetId="7" hidden="1">Hoja8!$E$8</definedName>
-    <definedName name="solver_lhs6" localSheetId="7" hidden="1">Hoja8!$E$9</definedName>
-    <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
-    <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_num" localSheetId="7" hidden="1">6</definedName>
-    <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="7" hidden="1">Hoja8!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
-    <definedName name="solver_rbv" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="7" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel5" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel6" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="7" hidden="1">Hoja8!$G$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="7" hidden="1">Hoja8!$G$11</definedName>
-    <definedName name="solver_rhs3" localSheetId="7" hidden="1">Hoja8!$G$6</definedName>
-    <definedName name="solver_rhs4" localSheetId="7" hidden="1">Hoja8!$G$7</definedName>
-    <definedName name="solver_rhs5" localSheetId="7" hidden="1">Hoja8!$G$8</definedName>
-    <definedName name="solver_rhs6" localSheetId="7" hidden="1">Hoja8!$G$9</definedName>
-    <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
-    <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
-    <definedName name="solver_typ" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="7" hidden="1">3</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="39">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
   <si>
-    <t xml:space="preserve">Tipo de carne</t>
+    <t>Tipo de carne</t>
   </si>
   <si>
     <t>R</t>
@@ -384,19 +401,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -410,21 +428,19 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -442,291 +458,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -917,17 +650,19 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -936,7 +671,7 @@
         <v>716.66666666666742</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -947,7 +682,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -958,7 +693,7 @@
         <v>0.41666666666666702</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -969,7 +704,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -977,15 +712,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="C9">
-        <v>0.32000000000000001</v>
+        <v>0.32</v>
       </c>
       <c r="D9">
         <f>B5*B9+C5*C9</f>
@@ -998,7 +733,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
@@ -1017,21 +752,20 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A2:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="12.7109375"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1040,7 +774,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1051,7 +785,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>20</v>
       </c>
@@ -1059,7 +793,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1070,12 +804,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>2</v>
       </c>
@@ -1093,7 +827,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
@@ -1111,7 +845,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>1</v>
       </c>
@@ -1127,18 +861,17 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1147,7 +880,7 @@
         <v>7.2727272727272751</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -1170,7 +903,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>0.90909090909090895</v>
       </c>
@@ -1190,7 +923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>2</v>
       </c>
@@ -1210,12 +943,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>20</v>
       </c>
@@ -1245,7 +978,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>50</v>
       </c>
@@ -1275,7 +1008,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>4</v>
       </c>
@@ -1306,18 +1039,17 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1326,7 +1058,7 @@
         <v>1250000</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -1343,7 +1075,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>50</v>
       </c>
@@ -1357,7 +1089,7 @@
         <v>9.9999999999999982</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>6000</v>
       </c>
@@ -1371,12 +1103,12 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>3</v>
       </c>
@@ -1400,7 +1132,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1424,7 +1156,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>2</v>
       </c>
@@ -1448,7 +1180,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E9">
         <v>1</v>
       </c>
@@ -1463,7 +1195,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>1</v>
       </c>
@@ -1478,7 +1210,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>1</v>
       </c>
@@ -1500,19 +1232,18 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>27</v>
       </c>
       <c r="B1">
@@ -1520,21 +1251,21 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>11.428571428571429</v>
       </c>
@@ -1545,7 +1276,7 @@
         <v>5.7142857142857144</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>700</v>
       </c>
@@ -1556,12 +1287,12 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>1</v>
       </c>
@@ -1575,14 +1306,14 @@
         <f>SUMPRODUCT(B3:D3,B6:D6)</f>
         <v>40</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="1">
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6">
         <v>40</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1593,14 +1324,14 @@
         <f>SUMPRODUCT(B3:C3,B7:C7)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>23</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>1</v>
       </c>
@@ -1611,7 +1342,7 @@
         <f>SUMPRODUCT(C3:D3,C8:D8)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" t="s">
         <v>23</v>
       </c>
       <c r="G8">
@@ -1619,50 +1350,40 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
       <c r="B1">
         <f>SUMPRODUCT(B3:D3,B4:D4)</f>
         <v>0</v>
       </c>
-      <c r="C1"/>
-      <c r="D1"/>
-      <c r="E1"/>
-      <c r="F1"/>
-      <c r="G1"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-    </row>
-    <row r="3">
-      <c r="A3"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>0</v>
       </c>
@@ -1672,12 +1393,8 @@
       <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3"/>
-      <c r="F3"/>
-      <c r="G3"/>
-    </row>
-    <row r="4">
-      <c r="A4"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1</v>
       </c>
@@ -1687,43 +1404,31 @@
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-    </row>
-    <row r="6">
-      <c r="A6"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6">
-        <v>0.20000000000000001</v>
-      </c>
-      <c r="C6"/>
+        <v>0.2</v>
+      </c>
       <c r="D6">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="E6">
         <f>B3*B6+D3*D6</f>
         <v>0</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" t="s">
         <v>9</v>
       </c>
       <c r="G6">
         <v>200</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7"/>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>0.5</v>
       </c>
@@ -1731,33 +1436,31 @@
         <v>0.5</v>
       </c>
       <c r="D7">
-        <v>0.40000000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="E7">
         <f>SUMPRODUCT($B$3:$D$3,B7:D7)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" t="s">
         <v>9</v>
       </c>
       <c r="G7">
         <v>800</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8"/>
-      <c r="B8"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="D8">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="E8">
         <f>SUMPRODUCT(C3:D3,C8:D8)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" t="s">
         <v>9</v>
       </c>
       <c r="G8">
@@ -1765,19 +1468,18 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>11</v>
       </c>
       <c r="B1">
@@ -1785,24 +1487,24 @@
         <v>33907636547.368427</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>0</v>
       </c>
@@ -1816,7 +1518,7 @@
         <v>8476909.1368421055</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>4000</v>
       </c>
@@ -1830,12 +1532,12 @@
         <v>-1000</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>1</v>
       </c>
@@ -1846,14 +1548,14 @@
         <f>SUMPRODUCT(B3:C3,B6:C6)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" t="s">
         <v>9</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D7">
         <v>6</v>
       </c>
@@ -1862,16 +1564,16 @@
       </c>
       <c r="F7">
         <f>SUMPRODUCT(D3:E3,D7:E7)</f>
-        <v>7.4505805969238281e-09</v>
-      </c>
-      <c r="G7" s="1" t="s">
+        <v>7.4505805969238281E-9</v>
+      </c>
+      <c r="G7" t="s">
         <v>9</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>2</v>
       </c>
@@ -1882,14 +1584,14 @@
         <f>SUMPRODUCT(B3:C3,B8:C8)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" t="s">
         <v>9</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D9">
         <v>2</v>
       </c>
@@ -1900,7 +1602,7 @@
         <f>SUMPRODUCT(D3:E3,D9:E9)</f>
         <v>-53687091.200000003</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" t="s">
         <v>9</v>
       </c>
       <c r="H9">
@@ -1908,41 +1610,40 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="1">
         <f>SUMPRODUCT(B3:D3,B4:D4)</f>
         <v>114999.99974829119</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>0.25000000755126428</v>
       </c>
@@ -1953,7 +1654,7 @@
         <v>2.2499999748291191</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>100000</v>
       </c>
@@ -1964,12 +1665,12 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>20000</v>
       </c>
@@ -1983,14 +1684,14 @@
         <f>SUMPRODUCT(B3:D3,B6:D6)</f>
         <v>18500</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="1">
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6">
         <v>18500</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>1</v>
       </c>
@@ -1998,14 +1699,14 @@
         <f>B3*B7</f>
         <v>0.25000000755126428</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>9</v>
       </c>
       <c r="G7">
         <v>10</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8">
         <v>1</v>
       </c>
@@ -2013,14 +1714,14 @@
         <f>C3*C8</f>
         <v>0</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" t="s">
         <v>9</v>
       </c>
       <c r="G8">
         <v>20</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D9">
         <v>1</v>
       </c>
@@ -2028,14 +1729,14 @@
         <f>D3*D9</f>
         <v>2.2499999748291191</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>9</v>
       </c>
       <c r="G9">
         <v>10</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>-0.5</v>
       </c>
@@ -2049,38 +1750,36 @@
         <f>SUMPRODUCT(B3:D3,B10:D10)</f>
         <v>-1.2499999911901916</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>0.90000000000000002</v>
+        <v>0.9</v>
       </c>
       <c r="C11">
-        <v>-0.10000000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="D11">
-        <v>-0.10000000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="E11">
         <f>SUMPRODUCT(B3:D3,B11:D11)</f>
-        <v>9.3132259404438145e-09</v>
-      </c>
-      <c r="F11" s="1" t="s">
+        <v>9.3132259404438145E-9</v>
+      </c>
+      <c r="F11" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-02 12:49:13
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="195" documentId="11_25ECF59304F7134D1C4F5E9C0BAFF804774F75A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{945858A0-6763-4ACD-AE07-CE3098277BCB}"/>
+  <xr:revisionPtr revIDLastSave="1015" documentId="11_25ECF59304F7134D1C4F5E9C0BAFF804774F75A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{680940ED-7E85-4B86-B6D0-E0B0451114C7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
@@ -140,10 +140,10 @@
     <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="5" hidden="1">0.0000001</definedName>
+    <definedName name="solver_pre" localSheetId="5" hidden="1">0.0000000000001</definedName>
     <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
-    <definedName name="solver_rbv" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="7" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
@@ -222,7 +222,7 @@
     <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="5" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
@@ -1418,7 +1418,7 @@
         <v>0.1</v>
       </c>
       <c r="E6">
-        <f>B3*B6+D3*D6</f>
+        <f>SUMPRODUCT(B3:D3,B6:D6)</f>
         <v>0</v>
       </c>
       <c r="F6" t="s">
@@ -1439,7 +1439,7 @@
         <v>0.4</v>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT($B$3:$D$3,B7:D7)</f>
+        <f>SUMPRODUCT(B3:D3,B7:D7)</f>
         <v>0</v>
       </c>
       <c r="F7" t="s">
@@ -1457,7 +1457,7 @@
         <v>0.3</v>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT(C3:D3,C8:D8)</f>
+        <f>SUMPRODUCT(B3:D3,B8:D8)</f>
         <v>0</v>
       </c>
       <c r="F8" t="s">

</xml_diff>

<commit_message>
vault backup: 2026-04-08 11:19:01
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,258 +8,275 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1015" documentId="11_25ECF59304F7134D1C4F5E9C0BAFF804774F75A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{680940ED-7E85-4B86-B6D0-E0B0451114C7}"/>
+  <xr:revisionPtr revIDLastSave="1320" documentId="11_25ECF59304F7134D1C4F5E9C0BAFF804774F75A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF3DE2B0-1B47-4B8E-A33B-F47AA7F14E15}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
-    <sheet name="Hoja5" sheetId="5" r:id="rId5"/>
-    <sheet name="Hoja6" sheetId="6" r:id="rId6"/>
-    <sheet name="Hoja7" sheetId="7" r:id="rId7"/>
-    <sheet name="Hoja8" sheetId="8" r:id="rId8"/>
+    <sheet name="Informe de respuestas 1" sheetId="9" r:id="rId1"/>
+    <sheet name="Informe de sensibilidad 1" sheetId="10" r:id="rId2"/>
+    <sheet name="Informe de límites 1" sheetId="11" r:id="rId3"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId4"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId5"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId6"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId7"/>
+    <sheet name="Hoja5" sheetId="5" r:id="rId8"/>
+    <sheet name="Hoja6" sheetId="6" r:id="rId9"/>
+    <sheet name="Hoja7" sheetId="7" r:id="rId10"/>
+    <sheet name="Hoja8" sheetId="8" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="solver_adj" localSheetId="0" hidden="1">Hoja1!$B$5:$C$5</definedName>
-    <definedName name="solver_adj" localSheetId="1" hidden="1">Hoja2!$B$5:$C$5</definedName>
-    <definedName name="solver_adj" localSheetId="2" hidden="1">Hoja3!$B$3:$G$3</definedName>
-    <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja4!$B$3:$E$3</definedName>
-    <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja5!$B$3:$D$3</definedName>
-    <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja6!$B$3:$D$3</definedName>
-    <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja7!$B$3:$E$3</definedName>
-    <definedName name="solver_adj" localSheetId="7" hidden="1">Hoja8!$B$3:$D$3</definedName>
-    <definedName name="solver_cvg" localSheetId="5" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="6" hidden="1">0.0001</definedName>
-    <definedName name="solver_cvg" localSheetId="7" hidden="1">0.0001</definedName>
-    <definedName name="solver_drv" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_drv" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_adj" localSheetId="3" hidden="1">Hoja1!$B$5:$C$5</definedName>
+    <definedName name="solver_adj" localSheetId="4" hidden="1">Hoja2!$B$5:$C$5</definedName>
+    <definedName name="solver_adj" localSheetId="5" hidden="1">Hoja3!$B$3:$G$3</definedName>
+    <definedName name="solver_adj" localSheetId="6" hidden="1">Hoja4!$B$3:$E$3</definedName>
+    <definedName name="solver_adj" localSheetId="7" hidden="1">Hoja5!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="8" hidden="1">Hoja6!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="9" hidden="1">Hoja7!$B$3:$E$3</definedName>
+    <definedName name="solver_adj" localSheetId="10" hidden="1">Hoja8!$B$3:$D$3</definedName>
+    <definedName name="solver_cvg" localSheetId="3" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="8" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="9" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="10" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_drv" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="10" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
-    <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
-    <definedName name="solver_eng" localSheetId="6" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="4" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="5" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="6" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="10" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_est" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_itr" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_est" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="10" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$D$9</definedName>
-    <definedName name="solver_lhs1" localSheetId="1" hidden="1">Hoja2!$D$9</definedName>
-    <definedName name="solver_lhs1" localSheetId="2" hidden="1">Hoja3!$H$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja4!$F$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja5!$E$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja6!$E$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja7!$F$6</definedName>
-    <definedName name="solver_lhs1" localSheetId="7" hidden="1">Hoja8!$E$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Hoja1!$D$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="1" hidden="1">Hoja2!$D$10</definedName>
-    <definedName name="solver_lhs2" localSheetId="2" hidden="1">Hoja3!$H$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja4!$F$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja5!$E$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja6!$E$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja7!$F$7</definedName>
-    <definedName name="solver_lhs2" localSheetId="7" hidden="1">Hoja8!$E$11</definedName>
-    <definedName name="solver_lhs3" localSheetId="1" hidden="1">Hoja2!$D$11</definedName>
-    <definedName name="solver_lhs3" localSheetId="2" hidden="1">Hoja3!$H$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="3" hidden="1">Hoja4!$F$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja5!$E$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja6!$E$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja7!$F$8</definedName>
-    <definedName name="solver_lhs3" localSheetId="7" hidden="1">Hoja8!$E$6</definedName>
-    <definedName name="solver_lhs4" localSheetId="3" hidden="1">Hoja4!$F$9</definedName>
-    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja7!$F$9</definedName>
-    <definedName name="solver_lhs4" localSheetId="7" hidden="1">Hoja8!$E$7</definedName>
-    <definedName name="solver_lhs5" localSheetId="3" hidden="1">Hoja4!$F$10</definedName>
-    <definedName name="solver_lhs5" localSheetId="7" hidden="1">Hoja8!$E$8</definedName>
-    <definedName name="solver_lhs6" localSheetId="3" hidden="1">Hoja4!$F$11</definedName>
-    <definedName name="solver_lhs6" localSheetId="7" hidden="1">Hoja8!$E$9</definedName>
-    <definedName name="solver_mip" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_mip" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_mni" localSheetId="5" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="6" hidden="1">30</definedName>
-    <definedName name="solver_mni" localSheetId="7" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="5" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="6" hidden="1">0.075</definedName>
-    <definedName name="solver_mrt" localSheetId="7" hidden="1">0.075</definedName>
-    <definedName name="solver_msl" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_msl" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_neg" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="9" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="10" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Hoja1!$D$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="4" hidden="1">Hoja2!$D$9</definedName>
+    <definedName name="solver_lhs1" localSheetId="5" hidden="1">Hoja3!$H$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="6" hidden="1">Hoja4!$F$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="7" hidden="1">Hoja5!$E$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="8" hidden="1">Hoja6!$E$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="9" hidden="1">Hoja7!$F$6</definedName>
+    <definedName name="solver_lhs1" localSheetId="10" hidden="1">Hoja8!$E$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Hoja1!$D$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="4" hidden="1">Hoja2!$D$10</definedName>
+    <definedName name="solver_lhs2" localSheetId="5" hidden="1">Hoja3!$H$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="6" hidden="1">Hoja4!$F$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="7" hidden="1">Hoja5!$E$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="8" hidden="1">Hoja6!$E$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="9" hidden="1">Hoja7!$F$7</definedName>
+    <definedName name="solver_lhs2" localSheetId="10" hidden="1">Hoja8!$E$11</definedName>
+    <definedName name="solver_lhs3" localSheetId="4" hidden="1">Hoja2!$D$11</definedName>
+    <definedName name="solver_lhs3" localSheetId="5" hidden="1">Hoja3!$H$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="6" hidden="1">Hoja4!$F$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="7" hidden="1">Hoja5!$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="8" hidden="1">Hoja6!$E$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="9" hidden="1">Hoja7!$F$8</definedName>
+    <definedName name="solver_lhs3" localSheetId="10" hidden="1">Hoja8!$E$6</definedName>
+    <definedName name="solver_lhs4" localSheetId="6" hidden="1">Hoja4!$F$9</definedName>
+    <definedName name="solver_lhs4" localSheetId="9" hidden="1">Hoja7!$F$9</definedName>
+    <definedName name="solver_lhs4" localSheetId="10" hidden="1">Hoja8!$E$7</definedName>
+    <definedName name="solver_lhs5" localSheetId="6" hidden="1">Hoja4!$F$10</definedName>
+    <definedName name="solver_lhs5" localSheetId="10" hidden="1">Hoja8!$E$8</definedName>
+    <definedName name="solver_lhs6" localSheetId="6" hidden="1">Hoja4!$F$11</definedName>
+    <definedName name="solver_lhs6" localSheetId="10" hidden="1">Hoja8!$E$9</definedName>
+    <definedName name="solver_mip" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="9" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="10" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="3" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="8" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="9" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="10" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="3" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="8" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="9" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="10" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="9" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="10" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="6" hidden="1">2147483647</definedName>
-    <definedName name="solver_nod" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_num" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="3" hidden="1">6</definedName>
+    <definedName name="solver_neg" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="3" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="9" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="10" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_num" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="5" hidden="1">3</definedName>
-    <definedName name="solver_num" localSheetId="6" hidden="1">4</definedName>
-    <definedName name="solver_num" localSheetId="7" hidden="1">6</definedName>
-    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="2" hidden="1">1</definedName>
+    <definedName name="solver_num" localSheetId="6" hidden="1">6</definedName>
+    <definedName name="solver_num" localSheetId="7" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="8" hidden="1">3</definedName>
+    <definedName name="solver_num" localSheetId="9" hidden="1">4</definedName>
+    <definedName name="solver_num" localSheetId="10" hidden="1">6</definedName>
     <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_nwt" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$B$2</definedName>
-    <definedName name="solver_opt" localSheetId="1" hidden="1">Hoja2!$B$2</definedName>
-    <definedName name="solver_opt" localSheetId="2" hidden="1">Hoja3!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja4!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja5!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja6!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja7!$B$1</definedName>
-    <definedName name="solver_opt" localSheetId="7" hidden="1">Hoja8!$B$1</definedName>
-    <definedName name="solver_pre" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_nwt" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="3" hidden="1">Hoja1!$B$2</definedName>
+    <definedName name="solver_opt" localSheetId="4" hidden="1">Hoja2!$B$2</definedName>
+    <definedName name="solver_opt" localSheetId="5" hidden="1">Hoja3!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="6" hidden="1">Hoja4!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="7" hidden="1">Hoja5!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="8" hidden="1">Hoja6!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="9" hidden="1">Hoja7!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="10" hidden="1">Hoja8!$B$1</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0</definedName>
-    <definedName name="solver_pre" localSheetId="5" hidden="1">0.0000000000001</definedName>
-    <definedName name="solver_pre" localSheetId="6" hidden="1">0.000001</definedName>
-    <definedName name="solver_pre" localSheetId="7" hidden="1">0.000001</definedName>
-    <definedName name="solver_rbv" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rbv" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rbv" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_pre" localSheetId="4" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="6" hidden="1">0</definedName>
+    <definedName name="solver_pre" localSheetId="8" hidden="1">0.0000000000001</definedName>
+    <definedName name="solver_pre" localSheetId="9" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="10" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rbv" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_rbv" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="10" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="4" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_rel2" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel2" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel2" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_rel2" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rel2" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="7" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="2" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="3" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="4" hidden="1">3</definedName>
-    <definedName name="solver_rel3" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="10" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="4" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="7" hidden="1">3</definedName>
+    <definedName name="solver_rel3" localSheetId="8" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="10" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_rel4" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel5" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_rel5" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rel6" localSheetId="3" hidden="1">3</definedName>
-    <definedName name="solver_rel6" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$9</definedName>
-    <definedName name="solver_rhs1" localSheetId="1" hidden="1">Hoja2!$F$9</definedName>
-    <definedName name="solver_rhs1" localSheetId="2" hidden="1">Hoja3!$J$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja4!$H$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja5!$G$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja6!$G$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja7!$H$6</definedName>
-    <definedName name="solver_rhs1" localSheetId="7" hidden="1">Hoja8!$G$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Hoja1!$F$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="1" hidden="1">Hoja2!$F$10</definedName>
-    <definedName name="solver_rhs2" localSheetId="2" hidden="1">Hoja3!$J$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja4!$H$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja5!$G$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja6!$G$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja7!$H$7</definedName>
-    <definedName name="solver_rhs2" localSheetId="7" hidden="1">Hoja8!$G$11</definedName>
-    <definedName name="solver_rhs3" localSheetId="1" hidden="1">Hoja2!$F$11</definedName>
-    <definedName name="solver_rhs3" localSheetId="2" hidden="1">Hoja3!$J$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="3" hidden="1">Hoja4!$H$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja5!$G$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja6!$G$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja7!$H$8</definedName>
-    <definedName name="solver_rhs3" localSheetId="7" hidden="1">Hoja8!$G$6</definedName>
-    <definedName name="solver_rhs4" localSheetId="3" hidden="1">Hoja4!$H$9</definedName>
-    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja7!$H$9</definedName>
-    <definedName name="solver_rhs4" localSheetId="7" hidden="1">Hoja8!$G$7</definedName>
-    <definedName name="solver_rhs5" localSheetId="3" hidden="1">Hoja4!$H$10</definedName>
-    <definedName name="solver_rhs5" localSheetId="7" hidden="1">Hoja8!$G$8</definedName>
-    <definedName name="solver_rhs6" localSheetId="3" hidden="1">Hoja4!$H$11</definedName>
-    <definedName name="solver_rhs6" localSheetId="7" hidden="1">Hoja8!$G$9</definedName>
-    <definedName name="solver_rlx" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_rlx" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_rsd" localSheetId="5" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="6" hidden="1">0</definedName>
-    <definedName name="solver_rsd" localSheetId="7" hidden="1">0</definedName>
-    <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_rel4" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="6" hidden="1">3</definedName>
+    <definedName name="solver_rel5" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_rel6" localSheetId="6" hidden="1">3</definedName>
+    <definedName name="solver_rel6" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Hoja1!$F$9</definedName>
+    <definedName name="solver_rhs1" localSheetId="4" hidden="1">Hoja2!$F$9</definedName>
+    <definedName name="solver_rhs1" localSheetId="5" hidden="1">Hoja3!$J$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="6" hidden="1">Hoja4!$H$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="7" hidden="1">Hoja5!$G$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="8" hidden="1">Hoja6!$G$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="9" hidden="1">Hoja7!$H$6</definedName>
+    <definedName name="solver_rhs1" localSheetId="10" hidden="1">Hoja8!$G$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Hoja1!$F$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="4" hidden="1">Hoja2!$F$10</definedName>
+    <definedName name="solver_rhs2" localSheetId="5" hidden="1">Hoja3!$J$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="6" hidden="1">Hoja4!$H$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="7" hidden="1">Hoja5!$G$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="8" hidden="1">Hoja6!$G$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="9" hidden="1">Hoja7!$H$7</definedName>
+    <definedName name="solver_rhs2" localSheetId="10" hidden="1">Hoja8!$G$11</definedName>
+    <definedName name="solver_rhs3" localSheetId="4" hidden="1">Hoja2!$F$11</definedName>
+    <definedName name="solver_rhs3" localSheetId="5" hidden="1">Hoja3!$J$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="6" hidden="1">Hoja4!$H$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="7" hidden="1">Hoja5!$G$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="8" hidden="1">Hoja6!$G$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="9" hidden="1">Hoja7!$H$8</definedName>
+    <definedName name="solver_rhs3" localSheetId="10" hidden="1">Hoja8!$G$6</definedName>
+    <definedName name="solver_rhs4" localSheetId="6" hidden="1">Hoja4!$H$9</definedName>
+    <definedName name="solver_rhs4" localSheetId="9" hidden="1">Hoja7!$H$9</definedName>
+    <definedName name="solver_rhs4" localSheetId="10" hidden="1">Hoja8!$G$7</definedName>
+    <definedName name="solver_rhs5" localSheetId="6" hidden="1">Hoja4!$H$10</definedName>
+    <definedName name="solver_rhs5" localSheetId="10" hidden="1">Hoja8!$G$8</definedName>
+    <definedName name="solver_rhs6" localSheetId="6" hidden="1">Hoja4!$H$11</definedName>
+    <definedName name="solver_rhs6" localSheetId="10" hidden="1">Hoja8!$G$9</definedName>
+    <definedName name="solver_rlx" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="9" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="10" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="3" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="8" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="9" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="10" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="4" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_scl" localSheetId="6" hidden="1">1</definedName>
-    <definedName name="solver_scl" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="6" hidden="1">2</definedName>
-    <definedName name="solver_sho" localSheetId="7" hidden="1">2</definedName>
-    <definedName name="solver_ssz" localSheetId="5" hidden="1">0</definedName>
-    <definedName name="solver_ssz" localSheetId="6" hidden="1">100</definedName>
-    <definedName name="solver_ssz" localSheetId="7" hidden="1">100</definedName>
-    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
-    <definedName name="solver_tim" localSheetId="2" hidden="1">2147483647</definedName>
+    <definedName name="solver_scl" localSheetId="6" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="10" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="3" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="9" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="10" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="2" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="3" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="8" hidden="1">0</definedName>
+    <definedName name="solver_ssz" localSheetId="9" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="10" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="5" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="6" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="7" hidden="1">2147483647</definedName>
-    <definedName name="solver_tol" localSheetId="5" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="6" hidden="1">0.01</definedName>
-    <definedName name="solver_tol" localSheetId="7" hidden="1">0.01</definedName>
-    <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
-    <definedName name="solver_typ" localSheetId="2" hidden="1">2</definedName>
-    <definedName name="solver_typ" localSheetId="3" hidden="1">1</definedName>
+    <definedName name="solver_tim" localSheetId="8" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="9" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="10" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="3" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="8" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="9" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="10" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="6" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="7" hidden="1">1</definedName>
-    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
-    <definedName name="solver_val" localSheetId="2" hidden="1">0</definedName>
+    <definedName name="solver_typ" localSheetId="8" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="9" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="10" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="6" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="7" hidden="1">0</definedName>
-    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
-    <definedName name="solver_ver" localSheetId="2" hidden="1">3</definedName>
+    <definedName name="solver_val" localSheetId="8" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="9" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="10" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="6" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="7" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="8" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="9" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="10" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -279,7 +296,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="94">
   <si>
     <t xml:space="preserve"> Costo</t>
   </si>
@@ -396,13 +413,178 @@
   </si>
   <si>
     <t>P</t>
+  </si>
+  <si>
+    <t>Microsoft Excel 16.0 Informe de respuestas</t>
+  </si>
+  <si>
+    <t>Hoja de cálculo: [TP3.xlsx]Hoja1</t>
+  </si>
+  <si>
+    <t>Informe creado: 8/4/2026 11:09:55</t>
+  </si>
+  <si>
+    <t>Resultado: Solver encontró una solución. Se cumplen todas las restricciones y condiciones óptimas.</t>
+  </si>
+  <si>
+    <t>Motor de Solver</t>
+  </si>
+  <si>
+    <t>Motor: Simplex LP</t>
+  </si>
+  <si>
+    <t>Tiempo de la solución: 0,016 segundos.</t>
+  </si>
+  <si>
+    <t>Iteraciones: 2 Subproblemas: 0</t>
+  </si>
+  <si>
+    <t>Opciones de Solver</t>
+  </si>
+  <si>
+    <t>Tiempo máximo Ilimitado,  Iteraciones Ilimitado, Precision 0</t>
+  </si>
+  <si>
+    <t>Máximo de subproblemas Ilimitado, Máximo de soluciones de enteros Ilimitado, Tolerancia de enteros 1%, Asumir no negativo</t>
+  </si>
+  <si>
+    <t>Celda objetivo (Mín)</t>
+  </si>
+  <si>
+    <t>Celda</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Valor original</t>
+  </si>
+  <si>
+    <t>Valor final</t>
+  </si>
+  <si>
+    <t>Celdas de variables</t>
+  </si>
+  <si>
+    <t>Entero</t>
+  </si>
+  <si>
+    <t>Valor de la celda</t>
+  </si>
+  <si>
+    <t>Fórmula</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Demora</t>
+  </si>
+  <si>
+    <t>$B$2</t>
+  </si>
+  <si>
+    <t>$B$5</t>
+  </si>
+  <si>
+    <t>cantidad R</t>
+  </si>
+  <si>
+    <t>Continuar</t>
+  </si>
+  <si>
+    <t>$C$5</t>
+  </si>
+  <si>
+    <t>cantidad C</t>
+  </si>
+  <si>
+    <t>$D$9</t>
+  </si>
+  <si>
+    <t>Grasa LI</t>
+  </si>
+  <si>
+    <t>$D$9&lt;=$F$9</t>
+  </si>
+  <si>
+    <t>Vinculante</t>
+  </si>
+  <si>
+    <t>$D$10</t>
+  </si>
+  <si>
+    <t>$D$10=$F$10</t>
+  </si>
+  <si>
+    <t>Microsoft Excel 16.0 Informe de sensibilidad</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Reducido</t>
+  </si>
+  <si>
+    <t>Coste</t>
+  </si>
+  <si>
+    <t>Objetivo</t>
+  </si>
+  <si>
+    <t>Coeficiente</t>
+  </si>
+  <si>
+    <t>Permisible</t>
+  </si>
+  <si>
+    <t>Aumentar</t>
+  </si>
+  <si>
+    <t>Reducir</t>
+  </si>
+  <si>
+    <t>Sombra</t>
+  </si>
+  <si>
+    <t>Precio</t>
+  </si>
+  <si>
+    <t>Restricción</t>
+  </si>
+  <si>
+    <t>Lado derecho</t>
+  </si>
+  <si>
+    <t>Microsoft Excel 16.0 Informe de límites</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Inferior</t>
+  </si>
+  <si>
+    <t>Límite</t>
+  </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>Superior</t>
+  </si>
+  <si>
+    <t>#N/D</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,6 +599,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -426,7 +624,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -434,13 +632,76 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="23"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="23"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="23"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="23"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="23"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="23"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="23"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,6 +717,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -655,11 +920,932 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AC737C2-60F1-46E0-BDD1-D05368465958}">
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6">
+        <v>716.66666666666742</v>
+      </c>
+      <c r="E16" s="6">
+        <v>716.66666666666663</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.58333333333333404</v>
+      </c>
+      <c r="E21" s="7">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="6">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="E22" s="6">
+        <v>0.41666666666666663</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G27" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="6">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1">
+        <f>SUMPRODUCT(B3:E3,B4:E4)</f>
+        <v>33907636547.368427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>7064090.9473684216</v>
+      </c>
+      <c r="E3">
+        <v>8476909.1368421055</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>4000</v>
+      </c>
+      <c r="C4">
+        <v>-3000</v>
+      </c>
+      <c r="D4">
+        <v>6000</v>
+      </c>
+      <c r="E4">
+        <v>-1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <f>SUMPRODUCT(B3:C3,B6:C6)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>-5</v>
+      </c>
+      <c r="F7">
+        <f>SUMPRODUCT(D3:E3,D7:E7)</f>
+        <v>7.4505805969238281E-9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>-8</v>
+      </c>
+      <c r="F8">
+        <f>SUMPRODUCT(B3:C3,B8:C8)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>-8</v>
+      </c>
+      <c r="F9">
+        <f>SUMPRODUCT(D3:E3,D9:E9)</f>
+        <v>-53687091.200000003</v>
+      </c>
+      <c r="G9" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1">
+        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
+        <v>114999.99974829119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>0.25000000755126428</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>2.2499999748291191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>100000</v>
+      </c>
+      <c r="C4">
+        <v>18000</v>
+      </c>
+      <c r="D4">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>20000</v>
+      </c>
+      <c r="C6">
+        <v>3000</v>
+      </c>
+      <c r="D6">
+        <v>6000</v>
+      </c>
+      <c r="E6">
+        <f>SUMPRODUCT(B3:D3,B6:D6)</f>
+        <v>18500</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6">
+        <v>18500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <f>B3*B7</f>
+        <v>0.25000000755126428</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <f>C3*C8</f>
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <f>D3*D9</f>
+        <v>2.2499999748291191</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>-0.5</v>
+      </c>
+      <c r="C10">
+        <v>0.5</v>
+      </c>
+      <c r="D10">
+        <v>-0.5</v>
+      </c>
+      <c r="E10">
+        <f>SUMPRODUCT(B3:D3,B10:D10)</f>
+        <v>-1.2499999911901916</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>0.9</v>
+      </c>
+      <c r="C11">
+        <v>-0.1</v>
+      </c>
+      <c r="D11">
+        <v>-0.1</v>
+      </c>
+      <c r="E11">
+        <f>SUMPRODUCT(B3:D3,B11:D11)</f>
+        <v>9.3132259404438145E-9</v>
+      </c>
+      <c r="F11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A1057C1-1458-41E5-9F81-2F95A0E94B20}">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>800</v>
+      </c>
+      <c r="G9" s="5">
+        <v>1E+30</v>
+      </c>
+      <c r="H9" s="5">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0.41666666666666663</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>600</v>
+      </c>
+      <c r="G10" s="3">
+        <v>200</v>
+      </c>
+      <c r="H10" s="3">
+        <v>1E+30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0.25</v>
+      </c>
+      <c r="E15" s="5">
+        <v>-1666.6666666666667</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0.25</v>
+      </c>
+      <c r="G15" s="5">
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="H15" s="5">
+        <v>4.9999999999999989E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1133.3333333333335</v>
+      </c>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0.24999999999999994</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0.21875</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4315D97D-C48A-4C8B-A0BC-DA273EC8F6A1}">
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.28515625" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="2.28515625" customWidth="1"/>
+    <col min="9" max="9" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="6">
+        <v>716.66666666666663</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="8"/>
+      <c r="C11" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="F11" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0.41666666666666663</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -668,7 +1854,7 @@
       </c>
       <c r="B2">
         <f>B5*B6+C5*C6</f>
-        <v>716.66666666666742</v>
+        <v>716.66666666666663</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -687,10 +1873,10 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.58333333333333404</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="C5">
-        <v>0.41666666666666702</v>
+        <v>0.41666666666666663</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -724,7 +1910,7 @@
       </c>
       <c r="D9">
         <f>B5*B9+C5*C9</f>
-        <v>0.25000000000000022</v>
+        <v>0.25</v>
       </c>
       <c r="E9" t="s">
         <v>9</v>
@@ -742,7 +1928,7 @@
       </c>
       <c r="D10">
         <f>B5*B10+C5*C10</f>
-        <v>1.0000000000000011</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
@@ -757,7 +1943,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -866,7 +2052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1044,7 +2230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1237,7 +2423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1355,7 +2541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1471,315 +2657,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1">
-        <f>SUMPRODUCT(B3:E3,B4:E4)</f>
-        <v>33907636547.368427</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>7064090.9473684216</v>
-      </c>
-      <c r="E3">
-        <v>8476909.1368421055</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>4000</v>
-      </c>
-      <c r="C4">
-        <v>-3000</v>
-      </c>
-      <c r="D4">
-        <v>6000</v>
-      </c>
-      <c r="E4">
-        <v>-1000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <f>SUMPRODUCT(B3:C3,B6:C6)</f>
-        <v>0</v>
-      </c>
-      <c r="G6" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D7">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>-5</v>
-      </c>
-      <c r="F7">
-        <f>SUMPRODUCT(D3:E3,D7:E7)</f>
-        <v>7.4505805969238281E-9</v>
-      </c>
-      <c r="G7" t="s">
-        <v>9</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8">
-        <v>-8</v>
-      </c>
-      <c r="F8">
-        <f>SUMPRODUCT(B3:C3,B8:C8)</f>
-        <v>0</v>
-      </c>
-      <c r="G8" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9">
-        <v>-8</v>
-      </c>
-      <c r="F9">
-        <f>SUMPRODUCT(D3:E3,D9:E9)</f>
-        <v>-53687091.200000003</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="1">
-        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
-        <v>114999.99974829119</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3">
-        <v>0.25000000755126428</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>2.2499999748291191</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>100000</v>
-      </c>
-      <c r="C4">
-        <v>18000</v>
-      </c>
-      <c r="D4">
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6">
-        <v>20000</v>
-      </c>
-      <c r="C6">
-        <v>3000</v>
-      </c>
-      <c r="D6">
-        <v>6000</v>
-      </c>
-      <c r="E6">
-        <f>SUMPRODUCT(B3:D3,B6:D6)</f>
-        <v>18500</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6">
-        <v>18500</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <f>B3*B7</f>
-        <v>0.25000000755126428</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <f>C3*C8</f>
-        <v>0</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <f>D3*D9</f>
-        <v>2.2499999748291191</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B10">
-        <v>-0.5</v>
-      </c>
-      <c r="C10">
-        <v>0.5</v>
-      </c>
-      <c r="D10">
-        <v>-0.5</v>
-      </c>
-      <c r="E10">
-        <f>SUMPRODUCT(B3:D3,B10:D10)</f>
-        <v>-1.2499999911901916</v>
-      </c>
-      <c r="F10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11">
-        <v>0.9</v>
-      </c>
-      <c r="C11">
-        <v>-0.1</v>
-      </c>
-      <c r="D11">
-        <v>-0.1</v>
-      </c>
-      <c r="E11">
-        <f>SUMPRODUCT(B3:D3,B11:D11)</f>
-        <v>9.3132259404438145E-9</v>
-      </c>
-      <c r="F11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-23 10:24:25
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4C8F10E-6E2E-40BD-9058-49B6996B05AD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="24" activeTab="29" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="6" activeTab="7" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -1785,30 +1785,27 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="16">
     <cellStyle name="Accent" xfId="1" xr:uid="{F7DA63D5-C2BB-44F7-AA68-DF2DD367A5E0}"/>
@@ -2416,10 +2413,10 @@
       <c r="F1" s="7"/>
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <f>B5*B6+C5*C6</f>
         <v>716.66666666666663</v>
       </c>
@@ -2437,13 +2434,13 @@
       <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>24</v>
       </c>
       <c r="D4" s="7"/>
@@ -2451,13 +2448,13 @@
       <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="8">
         <v>0.41666666666666663</v>
       </c>
       <c r="D5" s="7"/>
@@ -2465,13 +2462,13 @@
       <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="8">
         <v>800</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>600</v>
       </c>
       <c r="D6" s="7"/>
@@ -2487,54 +2484,54 @@
       <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="9"/>
+      <c r="B8" s="8"/>
       <c r="C8" s="7"/>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="8">
         <v>0.2</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="8">
         <v>0.32</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <f>SUMPRODUCT(B5:C5,B9:C9)</f>
         <v>0.25</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="8">
         <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9">
-        <v>1</v>
-      </c>
-      <c r="C10" s="9">
-        <v>1</v>
-      </c>
-      <c r="D10" s="9">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8">
+        <v>1</v>
+      </c>
+      <c r="C10" s="8">
+        <v>1</v>
+      </c>
+      <c r="D10" s="8">
         <f>SUMPRODUCT(B5:C5,B10:C10)</f>
         <v>1</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="8">
         <v>1</v>
       </c>
     </row>
@@ -2658,7 +2655,7 @@
       <c r="C8" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>7.2727272727272734</v>
       </c>
     </row>
@@ -2712,13 +2709,13 @@
       <c r="C13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>0.90909090909090906</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="3">
         <v>0.90909090909090828</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="3">
         <v>7.2727272727272716</v>
       </c>
       <c r="I13" s="3" t="s">
@@ -2735,13 +2732,13 @@
       <c r="C14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="3">
         <v>1.8181818181818183</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="3">
         <v>1.8181818181818181</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="3">
         <v>7.2727272727272725</v>
       </c>
       <c r="I14" s="3" t="s">
@@ -2758,13 +2755,13 @@
       <c r="C15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="12">
-        <v>0</v>
-      </c>
-      <c r="F15" s="12">
-        <v>0</v>
-      </c>
-      <c r="G15" s="12">
+      <c r="D15" s="3">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
         <v>7.2727272727272734</v>
       </c>
       <c r="I15" s="3" t="s">
@@ -2781,13 +2778,13 @@
       <c r="C16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="12">
-        <v>0</v>
-      </c>
-      <c r="F16" s="12">
-        <v>0</v>
-      </c>
-      <c r="G16" s="12">
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
         <v>7.2727272727272734</v>
       </c>
       <c r="I16" s="3" t="s">
@@ -2804,13 +2801,13 @@
       <c r="C17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D17" s="12">
-        <v>0</v>
-      </c>
-      <c r="F17" s="12">
-        <v>0</v>
-      </c>
-      <c r="G17" s="12">
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3">
         <v>7.2727272727272734</v>
       </c>
       <c r="I17" s="3" t="s">
@@ -2827,13 +2824,13 @@
       <c r="C18" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="11">
-        <v>0</v>
-      </c>
-      <c r="F18" s="11">
-        <v>0</v>
-      </c>
-      <c r="G18" s="11">
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4">
         <v>7.2727272727272734</v>
       </c>
       <c r="I18" s="4" t="s">
@@ -2926,16 +2923,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -2946,10 +2943,10 @@
       <c r="C16" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>7.2727272727272734</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>7.2727272727272734</v>
       </c>
     </row>
@@ -2959,19 +2956,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -2982,10 +2979,10 @@
       <c r="C21" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>0.90909090909090906</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>0.90909090909090906</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -2999,10 +2996,10 @@
       <c r="C22" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="3">
         <v>1.8181818181818183</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="3">
         <v>1.8181818181818183</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -3016,10 +3013,10 @@
       <c r="C23" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="12">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12">
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3">
         <v>0</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -3033,10 +3030,10 @@
       <c r="C24" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="12">
-        <v>0</v>
-      </c>
-      <c r="E24" s="12">
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3">
         <v>0</v>
       </c>
       <c r="F24" s="3" t="s">
@@ -3050,10 +3047,10 @@
       <c r="C25" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D25" s="12">
-        <v>0</v>
-      </c>
-      <c r="E25" s="12">
+      <c r="D25" s="3">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3">
         <v>0</v>
       </c>
       <c r="F25" s="3" t="s">
@@ -3067,10 +3064,10 @@
       <c r="C26" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D26" s="11">
-        <v>0</v>
-      </c>
-      <c r="E26" s="11">
+      <c r="D26" s="4">
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
         <v>0</v>
       </c>
       <c r="F26" s="4" t="s">
@@ -3083,22 +3080,22 @@
       </c>
     </row>
     <row r="30" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C30" s="10" t="s">
+      <c r="B30" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -3109,7 +3106,7 @@
       <c r="C31" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="3">
         <v>72.72727272727272</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -3118,7 +3115,7 @@
       <c r="F31" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="G31" s="12">
+      <c r="G31" s="3">
         <v>2.7272727272727195</v>
       </c>
     </row>
@@ -3129,7 +3126,7 @@
       <c r="C32" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="3">
         <v>100</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -3138,7 +3135,7 @@
       <c r="F32" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G32" s="12">
+      <c r="G32" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3149,7 +3146,7 @@
       <c r="C33" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="4">
         <v>20.000000000000004</v>
       </c>
       <c r="E33" s="4" t="s">
@@ -3158,7 +3155,7 @@
       <c r="F33" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="G33" s="11">
+      <c r="G33" s="4">
         <v>0</v>
       </c>
     </row>
@@ -3865,7 +3862,7 @@
       <c r="C8" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>1250000</v>
       </c>
     </row>
@@ -3919,19 +3916,19 @@
       <c r="C13" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>50</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="3">
         <v>50</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="3">
         <v>1250000</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="3">
         <v>50</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="3">
         <v>1250000</v>
       </c>
     </row>
@@ -3942,19 +3939,19 @@
       <c r="C14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="12">
-        <v>0</v>
-      </c>
-      <c r="F14" s="12">
-        <v>0</v>
-      </c>
-      <c r="G14" s="12">
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
         <v>1250000</v>
       </c>
-      <c r="I14" s="12">
-        <v>0</v>
-      </c>
-      <c r="J14" s="12">
+      <c r="I14" s="3">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3">
         <v>1250000</v>
       </c>
     </row>
@@ -3965,19 +3962,19 @@
       <c r="C15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="3">
         <v>145</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="3">
         <v>50</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="3">
         <v>680000</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="3">
         <v>145</v>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="3">
         <v>1250000</v>
       </c>
     </row>
@@ -3988,19 +3985,19 @@
       <c r="C16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>9.9999999999999947</v>
       </c>
-      <c r="F16" s="11">
-        <v>0</v>
-      </c>
-      <c r="G16" s="11">
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4">
         <v>1170000</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="4">
         <v>10</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="4">
         <v>1250000</v>
       </c>
     </row>
@@ -4087,16 +4084,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -4107,10 +4104,10 @@
       <c r="C16" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>1250000</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>1250000</v>
       </c>
     </row>
@@ -4120,19 +4117,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -4143,10 +4140,10 @@
       <c r="C21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>50</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>50</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -4160,10 +4157,10 @@
       <c r="C22" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="12">
-        <v>0</v>
-      </c>
-      <c r="E22" s="12">
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
         <v>0</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -4177,10 +4174,10 @@
       <c r="C23" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="3">
         <v>145</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="3">
         <v>145</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -4194,10 +4191,10 @@
       <c r="C24" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="4">
         <v>9.9999999999999947</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="4">
         <v>9.9999999999999947</v>
       </c>
       <c r="F24" s="4" t="s">
@@ -4210,22 +4207,22 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C28" s="10" t="s">
+      <c r="B28" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -4236,7 +4233,7 @@
       <c r="C29" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="3">
         <v>50</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -4245,7 +4242,7 @@
       <c r="F29" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4256,7 +4253,7 @@
       <c r="C30" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="3">
         <v>195</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -4265,7 +4262,7 @@
       <c r="F30" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="G30" s="12">
+      <c r="G30" s="3">
         <v>95</v>
       </c>
     </row>
@@ -4276,7 +4273,7 @@
       <c r="C31" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="3">
         <v>9.9999999999999947</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -4296,7 +4293,7 @@
       <c r="C32" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="3">
         <v>480</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -4316,7 +4313,7 @@
       <c r="C33" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="3">
         <v>400</v>
       </c>
       <c r="E33" s="3" t="s">
@@ -4336,7 +4333,7 @@
       <c r="C34" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D34" s="11">
+      <c r="D34" s="4">
         <v>370</v>
       </c>
       <c r="E34" s="4" t="s">
@@ -4990,16 +4987,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -5010,10 +5007,10 @@
       <c r="C16" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>40000</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>40000</v>
       </c>
     </row>
@@ -5023,19 +5020,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -5046,10 +5043,10 @@
       <c r="C21" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>11.428571428571431</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>11.428571428571431</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -5063,10 +5060,10 @@
       <c r="C22" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="3">
         <v>5.7142857142857153</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="3">
         <v>5.7142857142857153</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -5080,10 +5077,10 @@
       <c r="C23" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="4">
         <v>5.7142857142857135</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="4">
         <v>5.7142857142857135</v>
       </c>
       <c r="F23" s="4" t="s">
@@ -5096,22 +5093,22 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C27" s="10" t="s">
+      <c r="B27" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="G27" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -5122,7 +5119,7 @@
       <c r="C28" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="3">
         <v>0</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -5131,7 +5128,7 @@
       <c r="F28" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G28" s="12">
+      <c r="G28" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5142,7 +5139,7 @@
       <c r="C29" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="3">
         <v>1.7763568394002505E-15</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -5151,7 +5148,7 @@
       <c r="F29" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5162,7 +5159,7 @@
       <c r="C30" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="4">
         <v>40</v>
       </c>
       <c r="E30" s="4" t="s">
@@ -5238,7 +5235,7 @@
       <c r="C8" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>40000</v>
       </c>
     </row>
@@ -5292,19 +5289,19 @@
       <c r="C13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>11.428571428571431</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="3">
         <v>11.428571428571431</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="3">
         <v>40000</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="3">
         <v>11.428571428571431</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="3">
         <v>40000</v>
       </c>
     </row>
@@ -5315,19 +5312,19 @@
       <c r="C14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="3">
         <v>5.7142857142857153</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="3">
         <v>5.7142857142857135</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="3">
         <v>40000</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="3">
         <v>5.7142857142857135</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="3">
         <v>40000</v>
       </c>
     </row>
@@ -5338,19 +5335,19 @@
       <c r="C15" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="4">
         <v>5.7142857142857135</v>
       </c>
-      <c r="F15" s="11">
-        <v>0</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
         <v>20000.000000000004</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="4">
         <v>5.7142857142857126</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="4">
         <v>40000</v>
       </c>
     </row>
@@ -5417,7 +5414,7 @@
       <c r="C8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>716.66666666666663</v>
       </c>
     </row>
@@ -5471,7 +5468,7 @@
       <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>0.58333333333333337</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -5494,7 +5491,7 @@
       <c r="C14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="4">
         <v>0.41666666666666663</v>
       </c>
       <c r="F14" s="4" t="s">
@@ -5795,10 +5792,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="8">
+      <c r="B1" s="7">
         <f>SUMPRODUCT(B4:D4,B5:D5)</f>
         <v>1625</v>
       </c>
@@ -5818,16 +5815,16 @@
       <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>115</v>
       </c>
       <c r="E3" s="7"/>
@@ -5835,7 +5832,7 @@
       <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>116</v>
       </c>
       <c r="B4" s="7">
@@ -5867,87 +5864,87 @@
       <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="9"/>
+      <c r="B6" s="8"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <v>0.2</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>0.1</v>
       </c>
-      <c r="D7" s="9">
-        <v>0</v>
-      </c>
-      <c r="E7" s="9">
+      <c r="D7" s="8">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8">
         <f>SUMPRODUCT(B4:D4,B7:D7)</f>
         <v>200</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="8">
         <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="8">
         <v>0.5</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="8">
         <v>0.4</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="8">
         <v>0.5</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <f>SUMPRODUCT(B4:D4,B8:D8)</f>
         <v>800</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="8">
         <v>800</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="9">
-        <v>0</v>
-      </c>
-      <c r="C9" s="9">
+      <c r="B9" s="8">
+        <v>0</v>
+      </c>
+      <c r="C9" s="8">
         <v>0.30000000000000004</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>0.2</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <f>SUMPRODUCT(B4:D4,B9:D9)</f>
         <v>150.00000000000003</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="8">
         <v>150</v>
       </c>
     </row>
@@ -6080,7 +6077,7 @@
       <c r="C8" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>1625</v>
       </c>
     </row>
@@ -6134,7 +6131,7 @@
       <c r="C13" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>937.5</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -6143,10 +6140,10 @@
       <c r="G13" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="3">
         <v>937.49999999999989</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="3">
         <v>1625</v>
       </c>
     </row>
@@ -6157,7 +6154,7 @@
       <c r="C14" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="3">
         <v>125</v>
       </c>
       <c r="F14" s="3" t="s">
@@ -6166,10 +6163,10 @@
       <c r="G14" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="3">
         <v>124.99999999997158</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="3">
         <v>1624.9999999999718</v>
       </c>
     </row>
@@ -6180,7 +6177,7 @@
       <c r="C15" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="4">
         <v>562.50000000000011</v>
       </c>
       <c r="F15" s="4" t="s">
@@ -6189,10 +6186,10 @@
       <c r="G15" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="4">
         <v>562.49999999999204</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="4">
         <v>1624.999999999992</v>
       </c>
     </row>
@@ -6279,16 +6276,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -6299,10 +6296,10 @@
       <c r="C16" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>1625</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>1625</v>
       </c>
     </row>
@@ -6312,19 +6309,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -6335,10 +6332,10 @@
       <c r="C21" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>937.5</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>937.5</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -6352,10 +6349,10 @@
       <c r="C22" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="3">
         <v>125</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="3">
         <v>125</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -6369,10 +6366,10 @@
       <c r="C23" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="4">
         <v>562.50000000000011</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="4">
         <v>562.50000000000011</v>
       </c>
       <c r="F23" s="4" t="s">
@@ -6385,22 +6382,22 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C27" s="10" t="s">
+      <c r="B27" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="G27" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -6411,7 +6408,7 @@
       <c r="C28" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="3">
         <v>200</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -6431,7 +6428,7 @@
       <c r="C29" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="3">
         <v>800</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -6451,7 +6448,7 @@
       <c r="C30" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="4">
         <v>150.00000000000003</v>
       </c>
       <c r="E30" s="4" t="s">
@@ -6754,7 +6751,7 @@
       <c r="A1" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="8">
+      <c r="B1" s="7">
         <f>SUMPRODUCT(B4:E4,B5:E5)</f>
         <v>125000000</v>
       </c>
@@ -6891,7 +6888,7 @@
       <c r="E9" s="7">
         <v>0</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="7">
         <f>SUMPRODUCT(B4:E4,B9:E9)</f>
         <v>50000</v>
       </c>
@@ -6919,7 +6916,7 @@
       <c r="E10" s="7">
         <v>1</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="7">
         <f>SUMPRODUCT(B4:E4,B10:E10)</f>
         <v>5000</v>
       </c>
@@ -6947,7 +6944,7 @@
       <c r="E11" s="7">
         <v>0</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="7">
         <f>SUMPRODUCT(B4:E4,B11:E11)</f>
         <v>40000</v>
       </c>
@@ -6975,7 +6972,7 @@
       <c r="E12" s="7">
         <v>1</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="7">
         <f>SUMPRODUCT(B4:E4,B12:E12)</f>
         <v>15000</v>
       </c>
@@ -7003,7 +7000,7 @@
       <c r="E13" s="7">
         <v>0</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="7">
         <f>SUMPRODUCT(B4:E4,B13:E13)</f>
         <v>50000</v>
       </c>
@@ -7031,7 +7028,7 @@
       <c r="E14" s="7">
         <v>1</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="7">
         <f>SUMPRODUCT(B4:E4,B14:E14)</f>
         <v>5000</v>
       </c>
@@ -7059,7 +7056,7 @@
       <c r="E15" s="7">
         <v>0</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="7">
         <f>SUMPRODUCT(B4:E4,B15:E15)</f>
         <v>-40000</v>
       </c>
@@ -7087,7 +7084,7 @@
       <c r="E16" s="7">
         <v>-8</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="7">
         <f>SUMPRODUCT(B4:E4,B16:E16)</f>
         <v>0</v>
       </c>
@@ -7115,7 +7112,7 @@
       <c r="E17" s="7">
         <v>0</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="7">
         <f>SUMPRODUCT(B4:E4,B17:E17)</f>
         <v>104000</v>
       </c>
@@ -7143,7 +7140,7 @@
       <c r="E18" s="7">
         <v>5</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="7">
         <f>SUMPRODUCT(B4:E4,B18:E18)</f>
         <v>29000</v>
       </c>
@@ -7224,7 +7221,7 @@
       <c r="C8" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>125000000</v>
       </c>
     </row>
@@ -7278,19 +7275,19 @@
       <c r="C13" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>36000</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="3">
         <v>36000</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="3">
         <v>125000000</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="3">
         <v>36000</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="3">
         <v>125000000</v>
       </c>
     </row>
@@ -7301,19 +7298,19 @@
       <c r="C14" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="3">
         <v>14000</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="3">
         <v>14000</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="3">
         <v>125000000</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="3">
         <v>59000</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="3">
         <v>-10000000</v>
       </c>
     </row>
@@ -7324,19 +7321,19 @@
       <c r="C15" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="3">
         <v>4000</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="3">
         <v>4000</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="3">
         <v>125000000</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="3">
         <v>4000</v>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="3">
         <v>125000000</v>
       </c>
     </row>
@@ -7347,19 +7344,19 @@
       <c r="C16" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>1000</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="4">
         <v>1000</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="4">
         <v>125000000</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="4">
         <v>16000</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="4">
         <v>110000000</v>
       </c>
     </row>
@@ -7446,16 +7443,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -7466,10 +7463,10 @@
       <c r="C16" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>125000000</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>125000000</v>
       </c>
     </row>
@@ -7479,19 +7476,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -7502,10 +7499,10 @@
       <c r="C21" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>36000</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>36000</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -7519,10 +7516,10 @@
       <c r="C22" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="3">
         <v>14000</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="3">
         <v>14000</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -7536,10 +7533,10 @@
       <c r="C23" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="3">
         <v>4000</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="3">
         <v>4000</v>
       </c>
       <c r="F23" s="3" t="s">
@@ -7553,10 +7550,10 @@
       <c r="C24" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="4">
         <v>1000</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="4">
         <v>1000</v>
       </c>
       <c r="F24" s="4" t="s">
@@ -7569,22 +7566,22 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C28" s="10" t="s">
+      <c r="B28" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -7595,7 +7592,7 @@
       <c r="C29" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="3">
         <v>5000</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -7615,7 +7612,7 @@
       <c r="C30" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="3">
         <v>40000</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -7635,7 +7632,7 @@
       <c r="C31" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="3">
         <v>15000</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -7655,7 +7652,7 @@
       <c r="C32" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="3">
         <v>50000</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -7664,7 +7661,7 @@
       <c r="F32" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G32" s="12">
+      <c r="G32" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7675,7 +7672,7 @@
       <c r="C33" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="3">
         <v>5000</v>
       </c>
       <c r="E33" s="3" t="s">
@@ -7684,7 +7681,7 @@
       <c r="F33" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="G33" s="12">
+      <c r="G33" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7695,7 +7692,7 @@
       <c r="C34" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="3">
         <v>-40000</v>
       </c>
       <c r="E34" s="3" t="s">
@@ -7715,7 +7712,7 @@
       <c r="C35" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="3">
         <v>0</v>
       </c>
       <c r="E35" s="3" t="s">
@@ -7735,7 +7732,7 @@
       <c r="C36" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="3">
         <v>104000</v>
       </c>
       <c r="E36" s="3" t="s">
@@ -7744,7 +7741,7 @@
       <c r="F36" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="G36" s="12">
+      <c r="G36" s="3">
         <v>104000</v>
       </c>
     </row>
@@ -7755,7 +7752,7 @@
       <c r="C37" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="3">
         <v>29000</v>
       </c>
       <c r="E37" s="3" t="s">
@@ -7764,7 +7761,7 @@
       <c r="F37" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="G37" s="12">
+      <c r="G37" s="3">
         <v>29000</v>
       </c>
     </row>
@@ -7775,7 +7772,7 @@
       <c r="C38" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D38" s="11">
+      <c r="D38" s="4">
         <v>50000</v>
       </c>
       <c r="E38" s="4" t="s">
@@ -8260,7 +8257,7 @@
       <c r="A1" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="8">
+      <c r="B1" s="7">
         <f>SUMPRODUCT(B4:D4,B5:D5)</f>
         <v>123333.33333333333</v>
       </c>
@@ -8370,7 +8367,7 @@
       <c r="D8" s="7">
         <v>6000</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <f>SUMPRODUCT(B4:D4,B8:D8)</f>
         <v>18500</v>
       </c>
@@ -8395,7 +8392,7 @@
       <c r="D9" s="7">
         <v>0</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <f>SUMPRODUCT(B4:D4,B9:D9)</f>
         <v>0</v>
       </c>
@@ -8420,7 +8417,7 @@
       <c r="D10" s="7">
         <v>0</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <f>SUMPRODUCT(B4:D4,B10:D10)</f>
         <v>0</v>
       </c>
@@ -8445,7 +8442,7 @@
       <c r="D11" s="7">
         <v>1</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="7">
         <f>SUMPRODUCT(B4:D4,B11:D11)</f>
         <v>3.083333333333333</v>
       </c>
@@ -8470,7 +8467,7 @@
       <c r="D12" s="7">
         <v>-1</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="7">
         <f>SUMPRODUCT(B4:D4,B12:D12)</f>
         <v>-3.083333333333333</v>
       </c>
@@ -8495,7 +8492,7 @@
       <c r="D13" s="7">
         <v>1</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="7">
         <f>SUMPRODUCT(B4:D4,B13:D13)</f>
         <v>3.083333333333333</v>
       </c>
@@ -8606,16 +8603,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -8626,10 +8623,10 @@
       <c r="C16" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>716.66666666666663</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>716.66666666666663</v>
       </c>
     </row>
@@ -8639,19 +8636,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -8662,10 +8659,10 @@
       <c r="C21" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>0.58333333333333337</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -8679,10 +8676,10 @@
       <c r="C22" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="4">
         <v>0.41666666666666663</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="4">
         <v>0.41666666666666663</v>
       </c>
       <c r="F22" s="4" t="s">
@@ -8695,22 +8692,22 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C26" s="10" t="s">
+      <c r="B26" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -8721,7 +8718,7 @@
       <c r="C27" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="3">
         <v>0.25</v>
       </c>
       <c r="E27" s="3" t="s">
@@ -8741,7 +8738,7 @@
       <c r="C28" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="4">
         <v>1</v>
       </c>
       <c r="E28" s="4" t="s">
@@ -8817,7 +8814,7 @@
       <c r="C8" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>123333.33333333333</v>
       </c>
     </row>
@@ -8871,19 +8868,19 @@
       <c r="C13" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D13" s="12">
-        <v>0</v>
-      </c>
-      <c r="F13" s="12">
-        <v>0</v>
-      </c>
-      <c r="G13" s="12">
+      <c r="D13" s="3">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
         <v>123333.33333333333</v>
       </c>
-      <c r="I13" s="12">
-        <v>0</v>
-      </c>
-      <c r="J13" s="12">
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
         <v>123333.33333333333</v>
       </c>
     </row>
@@ -8894,19 +8891,19 @@
       <c r="C14" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D14" s="12">
-        <v>0</v>
-      </c>
-      <c r="F14" s="12">
-        <v>0</v>
-      </c>
-      <c r="G14" s="12">
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
         <v>123333.33333333333</v>
       </c>
-      <c r="I14" s="12">
-        <v>0</v>
-      </c>
-      <c r="J14" s="12">
+      <c r="I14" s="3">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3">
         <v>123333.33333333333</v>
       </c>
     </row>
@@ -8917,19 +8914,19 @@
       <c r="C15" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="4">
         <v>3.083333333333333</v>
       </c>
-      <c r="F15" s="11">
-        <v>0</v>
-      </c>
-      <c r="G15" s="11">
-        <v>0</v>
-      </c>
-      <c r="I15" s="11">
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4">
         <v>3.083333333333333</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="4">
         <v>123333.33333333333</v>
       </c>
     </row>
@@ -9016,16 +9013,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -9036,10 +9033,10 @@
       <c r="C16" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>123333.33333333333</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>123333.33333333333</v>
       </c>
     </row>
@@ -9049,19 +9046,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -9072,10 +9069,10 @@
       <c r="C21" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D21" s="12">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12">
+      <c r="D21" s="3">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3">
         <v>0</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -9089,10 +9086,10 @@
       <c r="C22" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D22" s="12">
-        <v>0</v>
-      </c>
-      <c r="E22" s="12">
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
         <v>0</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -9106,10 +9103,10 @@
       <c r="C23" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="4">
         <v>3.083333333333333</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="4">
         <v>3.083333333333333</v>
       </c>
       <c r="F23" s="4" t="s">
@@ -9122,22 +9119,22 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C27" s="10" t="s">
+      <c r="B27" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="G27" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -9148,7 +9145,7 @@
       <c r="C28" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="3">
         <v>0</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -9168,7 +9165,7 @@
       <c r="C29" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="3">
         <v>3.083333333333333</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -9188,7 +9185,7 @@
       <c r="C30" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="3">
         <v>-3.083333333333333</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -9208,7 +9205,7 @@
       <c r="C31" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="3">
         <v>3.083333333333333</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -9217,7 +9214,7 @@
       <c r="F31" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="G31" s="12">
+      <c r="G31" s="3">
         <v>3.083333333333333</v>
       </c>
     </row>
@@ -9228,7 +9225,7 @@
       <c r="C32" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="3">
         <v>18500</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -9248,7 +9245,7 @@
       <c r="C33" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="4">
         <v>0</v>
       </c>
       <c r="E33" s="4" t="s">
@@ -10739,7 +10736,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="4">
-        <v>1133.3333333333335</v>
+        <v>1133.3333333333301</v>
       </c>
       <c r="F16" s="4">
         <v>1</v>
@@ -10762,9 +10759,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="2.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5" customWidth="1"/>
+    <col min="3" max="3" width="6.625" customWidth="1"/>
+    <col min="4" max="4" width="8.5" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="3.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -11005,7 +11003,7 @@
       <c r="C8" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>180</v>
       </c>
     </row>
@@ -11059,19 +11057,19 @@
       <c r="C13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="3">
         <v>20</v>
       </c>
-      <c r="F13" s="12">
-        <v>0</v>
-      </c>
-      <c r="G13" s="12">
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
         <v>120</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="3">
         <v>20</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="3">
         <v>180</v>
       </c>
     </row>
@@ -11082,19 +11080,19 @@
       <c r="C14" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="4">
         <v>60</v>
       </c>
-      <c r="F14" s="11">
-        <v>0</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
         <v>60</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="4">
         <v>60</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="4">
         <v>180</v>
       </c>
     </row>
@@ -11181,16 +11179,16 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="B15" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>210</v>
       </c>
     </row>
@@ -11201,10 +11199,10 @@
       <c r="C16" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="4">
         <v>180</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="4">
         <v>180</v>
       </c>
     </row>
@@ -11214,19 +11212,19 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>211</v>
       </c>
     </row>
@@ -11237,10 +11235,10 @@
       <c r="C21" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="3">
         <v>20</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="3">
         <v>20</v>
       </c>
       <c r="F21" s="3" t="s">
@@ -11254,10 +11252,10 @@
       <c r="C22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="4">
         <v>60</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="4">
         <v>60</v>
       </c>
       <c r="F22" s="4" t="s">
@@ -11270,22 +11268,22 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C26" s="10" t="s">
+      <c r="B26" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="9" t="s">
         <v>215</v>
       </c>
     </row>
@@ -11296,7 +11294,7 @@
       <c r="C27" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="3">
         <v>20</v>
       </c>
       <c r="E27" s="3" t="s">
@@ -11316,7 +11314,7 @@
       <c r="C28" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="3">
         <v>100</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -11336,7 +11334,7 @@
       <c r="C29" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="4">
         <v>80</v>
       </c>
       <c r="E29" s="4" t="s">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 10:34:34
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4C8F10E-6E2E-40BD-9058-49B6996B05AD}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18F20BFA-6739-46AA-9E9C-FC4E20FA51BA}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="6" activeTab="7" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
   </bookViews>
@@ -1785,7 +1785,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1806,6 +1806,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="16">
     <cellStyle name="Accent" xfId="1" xr:uid="{F7DA63D5-C2BB-44F7-AA68-DF2DD367A5E0}"/>
@@ -11537,7 +11538,7 @@
       <c r="F15" s="3">
         <v>40</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="10">
         <v>1E+30</v>
       </c>
       <c r="H15" s="3">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 10:54:46
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18F20BFA-6739-46AA-9E9C-FC4E20FA51BA}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3FF448C-F9CA-4EC5-A1B7-422850776FF2}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="6" activeTab="7" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="32" activeTab="36" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -49,6 +49,8 @@
     <sheet name="Dual 1" sheetId="36" r:id="rId34"/>
     <sheet name="Primal 2" sheetId="35" r:id="rId35"/>
     <sheet name="Dual 2" sheetId="37" r:id="rId36"/>
+    <sheet name="Hoja2" sheetId="55" r:id="rId37"/>
+    <sheet name="Hoja3" sheetId="56" r:id="rId38"/>
   </sheets>
   <definedNames>
     <definedName name="solver_acr" localSheetId="16">0</definedName>
@@ -696,7 +698,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="288">
   <si>
     <t>Objetivo</t>
   </si>
@@ -1551,6 +1553,15 @@
   </si>
   <si>
     <t>$E$13&gt;=$G$13</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
 </sst>
 </file>
@@ -10534,6 +10545,41 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA11AE5B-9B4C-4E22-84EA-0C62D888AE05}">
+  <dimension ref="B2:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1E2C01-65FB-4999-9D74-801357ABBFE6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D582B61-11A9-4765-9151-155ECF620BD3}">
   <dimension ref="A1:H16"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 11:04:51
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3FF448C-F9CA-4EC5-A1B7-422850776FF2}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD768485-8C43-4D18-89C0-8047CB499371}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="32" activeTab="36" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
   </bookViews>
@@ -698,7 +698,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="289">
   <si>
     <t>Objetivo</t>
   </si>
@@ -1562,6 +1562,9 @@
   </si>
   <si>
     <t>L</t>
+  </si>
+  <si>
+    <t>&lt;</t>
   </si>
 </sst>
 </file>
@@ -10547,10 +10550,10 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA11AE5B-9B4C-4E22-84EA-0C62D888AE05}">
-  <dimension ref="B2:D4"/>
+  <dimension ref="B2:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>285</v>
       </c>
@@ -10561,9 +10564,79 @@
         <v>287</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4">
         <v>150</v>
+      </c>
+      <c r="C4">
+        <v>200</v>
+      </c>
+      <c r="D4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>288</v>
+      </c>
+      <c r="G7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>-1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>288</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>288</v>
+      </c>
+      <c r="G9">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="F10" t="s">
+        <v>288</v>
+      </c>
+      <c r="G10">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G11">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 11:14:55
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD768485-8C43-4D18-89C0-8047CB499371}"/>
+  <xr:revisionPtr revIDLastSave="684" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22F5B44F-6B36-45D0-95AB-02D249B3B55E}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="32" activeTab="36" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="35" activeTab="37" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -49,8 +49,12 @@
     <sheet name="Dual 1" sheetId="36" r:id="rId34"/>
     <sheet name="Primal 2" sheetId="35" r:id="rId35"/>
     <sheet name="Dual 2" sheetId="37" r:id="rId36"/>
-    <sheet name="Hoja2" sheetId="55" r:id="rId37"/>
-    <sheet name="Hoja3" sheetId="56" r:id="rId38"/>
+    <sheet name="EJ3" sheetId="55" r:id="rId37"/>
+    <sheet name="EJ3_B" sheetId="60" r:id="rId38"/>
+    <sheet name="Informe de respuestas 9" sheetId="57" r:id="rId39"/>
+    <sheet name="Informe de sensibilidad 9" sheetId="58" r:id="rId40"/>
+    <sheet name="Informe de límites 9" sheetId="59" r:id="rId41"/>
+    <sheet name="EJ4" sheetId="56" r:id="rId42"/>
   </sheets>
   <definedNames>
     <definedName name="solver_acr" localSheetId="16">0</definedName>
@@ -66,6 +70,8 @@
     <definedName name="solver_adj" localSheetId="28" hidden="1">'8'!$B$4:$D$4</definedName>
     <definedName name="solver_adj" localSheetId="33" hidden="1">'Dual 1'!$B$4:$E$4</definedName>
     <definedName name="solver_adj" localSheetId="35" hidden="1">'Dual 2'!$B$4:$D$4</definedName>
+    <definedName name="solver_adj" localSheetId="36" hidden="1">'EJ3'!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="37" hidden="1">EJ3_B!$B$3:$D$3</definedName>
     <definedName name="solver_adj" localSheetId="32" hidden="1">'Primal 1'!$B$4:$D$4</definedName>
     <definedName name="solver_adj" localSheetId="34" hidden="1">'Primal 2'!$B$4:$F$4</definedName>
     <definedName name="solver_adj_1" localSheetId="4">'2'!$B$3:$C$3</definedName>
@@ -96,6 +102,8 @@
     <definedName name="solver_cvg" localSheetId="28" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="33" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="35" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="36" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="37" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="32" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="34" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
@@ -108,6 +116,8 @@
     <definedName name="solver_drv" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_drv" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
@@ -120,6 +130,8 @@
     <definedName name="solver_eng" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="33" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="35" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="36" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="37" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_eng_1" localSheetId="4">2</definedName>
@@ -141,6 +153,8 @@
     <definedName name="solver_est" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_est_1" localSheetId="4">1</definedName>
@@ -162,6 +176,8 @@
     <definedName name="solver_itr" localSheetId="28" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="33" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="35" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="36" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="37" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_itr_1" localSheetId="4">2147483647</definedName>
@@ -183,6 +199,8 @@
     <definedName name="solver_lhs1" localSheetId="28" hidden="1">'8'!$E$10</definedName>
     <definedName name="solver_lhs1" localSheetId="33" hidden="1">'Dual 1'!$F$10</definedName>
     <definedName name="solver_lhs1" localSheetId="35" hidden="1">'Dual 2'!$E$10</definedName>
+    <definedName name="solver_lhs1" localSheetId="36" hidden="1">'EJ3'!$E$10</definedName>
+    <definedName name="solver_lhs1" localSheetId="37" hidden="1">EJ3_B!$E$10</definedName>
     <definedName name="solver_lhs1" localSheetId="32" hidden="1">'Primal 1'!$E$10</definedName>
     <definedName name="solver_lhs1" localSheetId="34" hidden="1">'Primal 2'!$G$10</definedName>
     <definedName name="solver_lhs1_1" localSheetId="4">'2'!$D$7</definedName>
@@ -199,6 +217,8 @@
     <definedName name="solver_lhs2" localSheetId="28" hidden="1">'8'!$E$11</definedName>
     <definedName name="solver_lhs2" localSheetId="33" hidden="1">'Dual 1'!$F$8</definedName>
     <definedName name="solver_lhs2" localSheetId="35" hidden="1">'Dual 2'!$E$11</definedName>
+    <definedName name="solver_lhs2" localSheetId="36" hidden="1">'EJ3'!$E$11</definedName>
+    <definedName name="solver_lhs2" localSheetId="37" hidden="1">EJ3_B!$E$11</definedName>
     <definedName name="solver_lhs2" localSheetId="32" hidden="1">'Primal 1'!$E$11</definedName>
     <definedName name="solver_lhs2" localSheetId="34" hidden="1">'Primal 2'!$G$8</definedName>
     <definedName name="solver_lhs2_1" localSheetId="4">'2'!$D$8</definedName>
@@ -213,6 +233,8 @@
     <definedName name="solver_lhs3" localSheetId="28" hidden="1">'8'!$E$12</definedName>
     <definedName name="solver_lhs3" localSheetId="33" hidden="1">'Dual 1'!$F$9</definedName>
     <definedName name="solver_lhs3" localSheetId="35" hidden="1">'Dual 2'!$E$12</definedName>
+    <definedName name="solver_lhs3" localSheetId="36" hidden="1">'EJ3'!$E$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="37" hidden="1">EJ3_B!$E$7</definedName>
     <definedName name="solver_lhs3" localSheetId="32" hidden="1">'Primal 1'!$E$8</definedName>
     <definedName name="solver_lhs3" localSheetId="34" hidden="1">'Primal 2'!$G$9</definedName>
     <definedName name="solver_lhs3_1" localSheetId="8">'3'!$H$9</definedName>
@@ -221,11 +243,15 @@
     <definedName name="solver_lhs4" localSheetId="24" hidden="1">'7'!$F$13</definedName>
     <definedName name="solver_lhs4" localSheetId="28" hidden="1">'8'!$E$13</definedName>
     <definedName name="solver_lhs4" localSheetId="35" hidden="1">'Dual 2'!$E$8</definedName>
+    <definedName name="solver_lhs4" localSheetId="36" hidden="1">'EJ3'!$E$8</definedName>
+    <definedName name="solver_lhs4" localSheetId="37" hidden="1">EJ3_B!$E$8</definedName>
     <definedName name="solver_lhs4" localSheetId="32" hidden="1">'Primal 1'!$E$9</definedName>
     <definedName name="solver_lhs5" localSheetId="12" hidden="1">'4'!$F$10</definedName>
     <definedName name="solver_lhs5" localSheetId="24" hidden="1">'7'!$F$14</definedName>
     <definedName name="solver_lhs5" localSheetId="28" hidden="1">'8'!$E$8</definedName>
     <definedName name="solver_lhs5" localSheetId="35" hidden="1">'Dual 2'!$E$9</definedName>
+    <definedName name="solver_lhs5" localSheetId="36" hidden="1">'EJ3'!$E$9</definedName>
+    <definedName name="solver_lhs5" localSheetId="37" hidden="1">EJ3_B!$E$9</definedName>
     <definedName name="solver_lhs6" localSheetId="12" hidden="1">'4'!$F$9</definedName>
     <definedName name="solver_lhs6" localSheetId="24" hidden="1">'7'!$F$15</definedName>
     <definedName name="solver_lhs6" localSheetId="28" hidden="1">'8'!$E$9</definedName>
@@ -251,6 +277,8 @@
     <definedName name="solver_mip" localSheetId="28" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="33" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="35" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="36" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="37" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
@@ -263,6 +291,8 @@
     <definedName name="solver_mni" localSheetId="28" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="33" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="35" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="36" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="37" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="32" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="34" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
@@ -275,6 +305,8 @@
     <definedName name="solver_mrt" localSheetId="28" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="33" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="35" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="36" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="37" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="32" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="34" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
@@ -287,6 +319,8 @@
     <definedName name="solver_msl" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="33" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="35" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="36" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="37" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_mtpb" localSheetId="16">0</definedName>
@@ -302,6 +336,8 @@
     <definedName name="solver_neg" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_neg_1" localSheetId="4">1</definedName>
@@ -317,6 +353,8 @@
     <definedName name="solver_nod" localSheetId="28" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="33" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="35" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="36" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="37" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
@@ -329,6 +367,8 @@
     <definedName name="solver_num" localSheetId="28" hidden="1">6</definedName>
     <definedName name="solver_num" localSheetId="33" hidden="1">3</definedName>
     <definedName name="solver_num" localSheetId="35" hidden="1">5</definedName>
+    <definedName name="solver_num" localSheetId="36" hidden="1">5</definedName>
+    <definedName name="solver_num" localSheetId="37" hidden="1">5</definedName>
     <definedName name="solver_num" localSheetId="32" hidden="1">4</definedName>
     <definedName name="solver_num" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_num_1" localSheetId="4">3</definedName>
@@ -344,6 +384,8 @@
     <definedName name="solver_nwt" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_nwt_1" localSheetId="4">1</definedName>
@@ -359,6 +401,8 @@
     <definedName name="solver_opt" localSheetId="28" hidden="1">'8'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="33" hidden="1">'Dual 1'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="35" hidden="1">'Dual 2'!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="36" hidden="1">'EJ3'!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="37" hidden="1">EJ3_B!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="32" hidden="1">'Primal 1'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="34" hidden="1">'Primal 2'!$B$1</definedName>
     <definedName name="solver_opt_1" localSheetId="4">'2'!$B$1</definedName>
@@ -374,6 +418,8 @@
     <definedName name="solver_pre" localSheetId="28" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="33" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="35" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="36" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="37" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="32" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="34" hidden="1">0.000001</definedName>
     <definedName name="solver_pre_1" localSheetId="4">0</definedName>
@@ -392,6 +438,8 @@
     <definedName name="solver_rbv" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_rbv" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
@@ -404,6 +452,8 @@
     <definedName name="solver_rel1" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_rel1_1" localSheetId="4">1</definedName>
@@ -420,6 +470,8 @@
     <definedName name="solver_rel2" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_rel2_1" localSheetId="4">1</definedName>
@@ -434,6 +486,8 @@
     <definedName name="solver_rel3" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_rel3_1" localSheetId="8">3</definedName>
@@ -442,11 +496,15 @@
     <definedName name="solver_rel4" localSheetId="24" hidden="1">3</definedName>
     <definedName name="solver_rel4" localSheetId="28" hidden="1">3</definedName>
     <definedName name="solver_rel4" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel5" localSheetId="12" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="24" hidden="1">3</definedName>
     <definedName name="solver_rel5" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="12" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="24" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="28" hidden="1">1</definedName>
@@ -464,6 +522,8 @@
     <definedName name="solver_rhs1" localSheetId="28" hidden="1">'8'!$G$10</definedName>
     <definedName name="solver_rhs1" localSheetId="33" hidden="1">'Dual 1'!$H$10</definedName>
     <definedName name="solver_rhs1" localSheetId="35" hidden="1">'Dual 2'!$G$10</definedName>
+    <definedName name="solver_rhs1" localSheetId="36" hidden="1">'EJ3'!$G$10</definedName>
+    <definedName name="solver_rhs1" localSheetId="37" hidden="1">EJ3_B!$G$10</definedName>
     <definedName name="solver_rhs1" localSheetId="32" hidden="1">'Primal 1'!$G$10</definedName>
     <definedName name="solver_rhs1" localSheetId="34" hidden="1">'Primal 2'!$I$10</definedName>
     <definedName name="solver_rhs1_1" localSheetId="4">'2'!$F$7</definedName>
@@ -480,6 +540,8 @@
     <definedName name="solver_rhs2" localSheetId="28" hidden="1">'8'!$G$11</definedName>
     <definedName name="solver_rhs2" localSheetId="33" hidden="1">'Dual 1'!$H$8</definedName>
     <definedName name="solver_rhs2" localSheetId="35" hidden="1">'Dual 2'!$G$11</definedName>
+    <definedName name="solver_rhs2" localSheetId="36" hidden="1">'EJ3'!$G$11</definedName>
+    <definedName name="solver_rhs2" localSheetId="37" hidden="1">EJ3_B!$G$11</definedName>
     <definedName name="solver_rhs2" localSheetId="32" hidden="1">'Primal 1'!$G$11</definedName>
     <definedName name="solver_rhs2" localSheetId="34" hidden="1">'Primal 2'!$I$8</definedName>
     <definedName name="solver_rhs2_1" localSheetId="4">'2'!$F$8</definedName>
@@ -494,6 +556,8 @@
     <definedName name="solver_rhs3" localSheetId="28" hidden="1">'8'!$G$12</definedName>
     <definedName name="solver_rhs3" localSheetId="33" hidden="1">'Dual 1'!$H$9</definedName>
     <definedName name="solver_rhs3" localSheetId="35" hidden="1">'Dual 2'!$G$12</definedName>
+    <definedName name="solver_rhs3" localSheetId="36" hidden="1">'EJ3'!$G$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="37" hidden="1">EJ3_B!$G$7</definedName>
     <definedName name="solver_rhs3" localSheetId="32" hidden="1">'Primal 1'!$G$8</definedName>
     <definedName name="solver_rhs3" localSheetId="34" hidden="1">'Primal 2'!$I$9</definedName>
     <definedName name="solver_rhs3_1" localSheetId="8">'3'!$J$9</definedName>
@@ -502,11 +566,15 @@
     <definedName name="solver_rhs4" localSheetId="24" hidden="1">'7'!$H$13</definedName>
     <definedName name="solver_rhs4" localSheetId="28" hidden="1">'8'!$G$13</definedName>
     <definedName name="solver_rhs4" localSheetId="35" hidden="1">'Dual 2'!$G$8</definedName>
+    <definedName name="solver_rhs4" localSheetId="36" hidden="1">'EJ3'!$G$8</definedName>
+    <definedName name="solver_rhs4" localSheetId="37" hidden="1">EJ3_B!$G$8</definedName>
     <definedName name="solver_rhs4" localSheetId="32" hidden="1">'Primal 1'!$G$9</definedName>
     <definedName name="solver_rhs5" localSheetId="12" hidden="1">'4'!$H$10</definedName>
     <definedName name="solver_rhs5" localSheetId="24" hidden="1">'7'!$H$14</definedName>
     <definedName name="solver_rhs5" localSheetId="28" hidden="1">'8'!$G$8</definedName>
     <definedName name="solver_rhs5" localSheetId="35" hidden="1">'Dual 2'!$G$9</definedName>
+    <definedName name="solver_rhs5" localSheetId="36" hidden="1">'EJ3'!$G$9</definedName>
+    <definedName name="solver_rhs5" localSheetId="37" hidden="1">EJ3_B!$G$9</definedName>
     <definedName name="solver_rhs6" localSheetId="12" hidden="1">'4'!$H$9</definedName>
     <definedName name="solver_rhs6" localSheetId="24" hidden="1">'7'!$H$15</definedName>
     <definedName name="solver_rhs6" localSheetId="28" hidden="1">'8'!$G$9</definedName>
@@ -524,6 +592,8 @@
     <definedName name="solver_rlx" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="33" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="35" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="36" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="37" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
@@ -536,6 +606,8 @@
     <definedName name="solver_rsd" localSheetId="28" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="33" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="35" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="36" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="37" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="32" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="34" hidden="1">0</definedName>
     <definedName name="solver_rsp" localSheetId="16">0</definedName>
@@ -551,6 +623,8 @@
     <definedName name="solver_scl" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_scl_1" localSheetId="4">1</definedName>
@@ -566,6 +640,8 @@
     <definedName name="solver_sho" localSheetId="28" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="33" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="35" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="36" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="37" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="9" hidden="1">2</definedName>
@@ -574,6 +650,7 @@
     <definedName name="solver_sho" localSheetId="21" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="25" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="29" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="40" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_slim" localSheetId="16">70</definedName>
@@ -598,6 +675,8 @@
     <definedName name="solver_ssz" localSheetId="28" hidden="1">70</definedName>
     <definedName name="solver_ssz" localSheetId="33" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="35" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="36" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="37" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="32" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="34" hidden="1">100</definedName>
     <definedName name="solver_stol" localSheetId="16">0.000001</definedName>
@@ -613,6 +692,8 @@
     <definedName name="solver_tim" localSheetId="28" hidden="1">60000</definedName>
     <definedName name="solver_tim" localSheetId="33" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="35" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="36" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="37" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_tim_1" localSheetId="4">2147483647</definedName>
@@ -628,6 +709,8 @@
     <definedName name="solver_tol" localSheetId="28" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="33" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="35" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="36" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="37" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="32" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="34" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
@@ -640,6 +723,8 @@
     <definedName name="solver_typ" localSheetId="28" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="33" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="35" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="36" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="37" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_typ_1" localSheetId="4">1</definedName>
@@ -655,6 +740,8 @@
     <definedName name="solver_val" localSheetId="28" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="33" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="35" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="36" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="37" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="32" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="34" hidden="1">0</definedName>
     <definedName name="solver_val_1" localSheetId="4">0</definedName>
@@ -670,6 +757,8 @@
     <definedName name="solver_ver" localSheetId="28" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="33" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="35" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="36" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="37" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_ver_1" localSheetId="4">3</definedName>
@@ -698,7 +787,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="291">
   <si>
     <t>Objetivo</t>
   </si>
@@ -1565,6 +1654,12 @@
   </si>
   <si>
     <t>&lt;</t>
+  </si>
+  <si>
+    <t>Hoja de cálculo: [TP3.xlsx]EJ3</t>
+  </si>
+  <si>
+    <t>Informe creado: 23/4/2026 11:08:58</t>
   </si>
 </sst>
 </file>
@@ -1799,7 +1894,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1821,6 +1916,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="16">
     <cellStyle name="Accent" xfId="1" xr:uid="{F7DA63D5-C2BB-44F7-AA68-DF2DD367A5E0}"/>
@@ -10550,9 +10658,21 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA11AE5B-9B4C-4E22-84EA-0C62D888AE05}">
-  <dimension ref="B2:G11"/>
+  <dimension ref="B1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.75" customWidth="1"/>
+    <col min="7" max="7" width="3.875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
+    <row r="1" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B1">
+        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
+        <v>4250</v>
+      </c>
+    </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>285</v>
@@ -10564,6 +10684,17 @@
         <v>287</v>
       </c>
     </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>25.000000000000004</v>
+      </c>
+      <c r="C3">
+        <v>19.999999999999996</v>
+      </c>
+      <c r="D3">
+        <v>350</v>
+      </c>
+    </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4">
         <v>150</v>
@@ -10582,6 +10713,10 @@
       <c r="C7">
         <v>1</v>
       </c>
+      <c r="E7">
+        <f>SUMPRODUCT(B7:D7,B3:D3)</f>
+        <v>45</v>
+      </c>
       <c r="F7" t="s">
         <v>288</v>
       </c>
@@ -10599,6 +10734,10 @@
       <c r="D8">
         <v>-1</v>
       </c>
+      <c r="E8">
+        <f>SUMPRODUCT(B3:D3,B8:D8)</f>
+        <v>0</v>
+      </c>
       <c r="F8" t="s">
         <v>288</v>
       </c>
@@ -10609,6 +10748,10 @@
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="D9">
         <v>1</v>
+      </c>
+      <c r="E9">
+        <f>SUMPRODUCT(B3:D3,B9:D9)</f>
+        <v>350</v>
       </c>
       <c r="F9" t="s">
         <v>288</v>
@@ -10621,6 +10764,10 @@
       <c r="B10">
         <v>5</v>
       </c>
+      <c r="E10">
+        <f>SUMPRODUCT(B3:D3,B10:D10)</f>
+        <v>125.00000000000001</v>
+      </c>
       <c r="F10" t="s">
         <v>288</v>
       </c>
@@ -10631,6 +10778,10 @@
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C11">
         <v>4</v>
+      </c>
+      <c r="E11">
+        <f>SUMPRODUCT(B3:D3,B11:D11)</f>
+        <v>79.999999999999986</v>
       </c>
       <c r="F11" t="s">
         <v>288</v>
@@ -10645,10 +10796,430 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1E2C01-65FB-4999-9D74-801357ABBFE6}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276FD171-69C1-4A34-931E-4257BD858AE0}">
+  <dimension ref="B1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B1">
+        <f>SUMPRODUCT(B3:D3,B4:D4)</f>
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>25.000000000000004</v>
+      </c>
+      <c r="C3">
+        <v>19.999999999999996</v>
+      </c>
+      <c r="D3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>130</v>
+      </c>
+      <c r="C4">
+        <v>200</v>
+      </c>
+      <c r="D4">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <f>SUMPRODUCT(B7:D7,B3:D3)</f>
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>288</v>
+      </c>
+      <c r="G7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>-1</v>
+      </c>
+      <c r="E8">
+        <f>SUMPRODUCT(B3:D3,B8:D8)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>288</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <f>SUMPRODUCT(B3:D3,B9:D9)</f>
+        <v>350</v>
+      </c>
+      <c r="F9" t="s">
+        <v>288</v>
+      </c>
+      <c r="G9">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <f>SUMPRODUCT(B3:D3,B10:D10)</f>
+        <v>125.00000000000001</v>
+      </c>
+      <c r="F10" t="s">
+        <v>288</v>
+      </c>
+      <c r="G10">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <f>SUMPRODUCT(B3:D3,B11:D11)</f>
+        <v>79.999999999999986</v>
+      </c>
+      <c r="F11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G11">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFEFA73-1A95-4AFE-97FB-0E74D240D17A}">
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.125" customWidth="1"/>
+    <col min="2" max="2" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="14">
+        <v>0</v>
+      </c>
+      <c r="E16" s="14">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D21" s="15">
+        <v>0</v>
+      </c>
+      <c r="E21" s="15">
+        <v>25.000000000000004</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B22" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D22" s="15">
+        <v>0</v>
+      </c>
+      <c r="E22" s="15">
+        <v>19.999999999999996</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="D23" s="14">
+        <v>0</v>
+      </c>
+      <c r="E23" s="14">
+        <v>350</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B28" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="15">
+        <v>125.00000000000001</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="G28" s="13">
+        <v>14.999999999999986</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B29" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="15">
+        <v>79.999999999999986</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="G29" s="13">
+        <v>40.000000000000014</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="15">
+        <v>45</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G30" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="15">
+        <v>0</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G31" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" s="11"/>
+      <c r="D32" s="14">
+        <v>350</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G32" s="11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10869,6 +11440,495 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD391165-EA5C-4F0E-A10D-4A06AF2C0A78}">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.125" customWidth="1"/>
+    <col min="2" max="2" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B9" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D9" s="13">
+        <v>25.000000000000004</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <v>150</v>
+      </c>
+      <c r="G9" s="13">
+        <v>10.000000000000018</v>
+      </c>
+      <c r="H9" s="13">
+        <v>29.999999999999982</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B10" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D10" s="13">
+        <v>19.999999999999996</v>
+      </c>
+      <c r="E10" s="13">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <v>200</v>
+      </c>
+      <c r="G10" s="13">
+        <v>49.999999999999964</v>
+      </c>
+      <c r="H10" s="13">
+        <v>10.000000000000018</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="D11" s="11">
+        <v>350</v>
+      </c>
+      <c r="E11" s="11">
+        <v>0</v>
+      </c>
+      <c r="F11" s="11">
+        <v>-10</v>
+      </c>
+      <c r="G11" s="11">
+        <v>1E+30</v>
+      </c>
+      <c r="H11" s="11">
+        <v>2.5000000000000049</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B16" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13">
+        <v>125.00000000000001</v>
+      </c>
+      <c r="E16" s="13">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13">
+        <v>140</v>
+      </c>
+      <c r="G16" s="13">
+        <v>1E+30</v>
+      </c>
+      <c r="H16" s="13">
+        <v>15.000000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B17" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13">
+        <v>79.999999999999986</v>
+      </c>
+      <c r="E17" s="13">
+        <v>0</v>
+      </c>
+      <c r="F17" s="13">
+        <v>120</v>
+      </c>
+      <c r="G17" s="13">
+        <v>1E+30</v>
+      </c>
+      <c r="H17" s="13">
+        <v>40.000000000000014</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B18" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13">
+        <v>45</v>
+      </c>
+      <c r="E18" s="13">
+        <v>74.999999999999972</v>
+      </c>
+      <c r="F18" s="13">
+        <v>45</v>
+      </c>
+      <c r="G18" s="13">
+        <v>1.2000000000000002</v>
+      </c>
+      <c r="H18" s="13">
+        <v>6.666666666666667</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B19" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13">
+        <v>0</v>
+      </c>
+      <c r="E19" s="13">
+        <v>12.500000000000005</v>
+      </c>
+      <c r="F19" s="13">
+        <v>0</v>
+      </c>
+      <c r="G19" s="13">
+        <v>40.000000000000007</v>
+      </c>
+      <c r="H19" s="13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11">
+        <v>350</v>
+      </c>
+      <c r="E20" s="11">
+        <v>2.5000000000000049</v>
+      </c>
+      <c r="F20" s="11">
+        <v>350</v>
+      </c>
+      <c r="G20" s="11">
+        <v>40.000000000000007</v>
+      </c>
+      <c r="H20" s="11">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89867AE7-940A-4F7C-B8F3-D6C17C5ADF23}">
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.125" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.125" customWidth="1"/>
+    <col min="6" max="6" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="2.125" customWidth="1"/>
+    <col min="9" max="9" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="B6" s="16"/>
+      <c r="C6" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="14">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="B11" s="16"/>
+      <c r="C11" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="F11" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B13" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D13" s="15">
+        <v>25.000000000000004</v>
+      </c>
+      <c r="F13" s="15">
+        <v>0</v>
+      </c>
+      <c r="G13" s="15">
+        <v>499.99999999999909</v>
+      </c>
+      <c r="I13" s="15">
+        <v>25.000000000000004</v>
+      </c>
+      <c r="J13" s="15">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D14" s="15">
+        <v>19.999999999999996</v>
+      </c>
+      <c r="F14" s="15">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15">
+        <v>250.00000000000045</v>
+      </c>
+      <c r="I14" s="15">
+        <v>20</v>
+      </c>
+      <c r="J14" s="15">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="D15" s="14">
+        <v>350</v>
+      </c>
+      <c r="F15" s="14">
+        <v>350</v>
+      </c>
+      <c r="G15" s="14">
+        <v>4250</v>
+      </c>
+      <c r="I15" s="14">
+        <v>350</v>
+      </c>
+      <c r="J15" s="14">
+        <v>4250</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1E2C01-65FB-4999-9D74-801357ABBFE6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 11:35:06
</commit_message>
<xml_diff>
--- a/Materias/4to/Investigacion operativa/Material/TP3.xlsx
+++ b/Materias/4to/Investigacion operativa/Material/TP3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81c81c830e246c0e/Escritorio/Facultad/Obsidian/Vault_Obsidian/Materias/4to/Investigacion operativa/Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="684" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22F5B44F-6B36-45D0-95AB-02D249B3B55E}"/>
+  <xr:revisionPtr revIDLastSave="1325" documentId="13_ncr:8000000b_{98C0940C-457F-4AA0-B8E5-18007E51AF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2591E943-0545-437F-9D37-B584EA643DA0}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="35" activeTab="37" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="41" activeTab="42" xr2:uid="{A43AA329-DB2E-4710-B187-C60C5E009D8A}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -55,6 +55,9 @@
     <sheet name="Informe de sensibilidad 9" sheetId="58" r:id="rId40"/>
     <sheet name="Informe de límites 9" sheetId="59" r:id="rId41"/>
     <sheet name="EJ4" sheetId="56" r:id="rId42"/>
+    <sheet name="Informe de respuestas 10" sheetId="61" r:id="rId43"/>
+    <sheet name="Informe de sensibilidad 10" sheetId="62" r:id="rId44"/>
+    <sheet name="Informe de límites 10" sheetId="63" r:id="rId45"/>
   </sheets>
   <definedNames>
     <definedName name="solver_acr" localSheetId="16">0</definedName>
@@ -72,6 +75,7 @@
     <definedName name="solver_adj" localSheetId="35" hidden="1">'Dual 2'!$B$4:$D$4</definedName>
     <definedName name="solver_adj" localSheetId="36" hidden="1">'EJ3'!$B$3:$D$3</definedName>
     <definedName name="solver_adj" localSheetId="37" hidden="1">EJ3_B!$B$3:$D$3</definedName>
+    <definedName name="solver_adj" localSheetId="41" hidden="1">'EJ4'!$B$4:$G$4</definedName>
     <definedName name="solver_adj" localSheetId="32" hidden="1">'Primal 1'!$B$4:$D$4</definedName>
     <definedName name="solver_adj" localSheetId="34" hidden="1">'Primal 2'!$B$4:$F$4</definedName>
     <definedName name="solver_adj_1" localSheetId="4">'2'!$B$3:$C$3</definedName>
@@ -104,6 +108,7 @@
     <definedName name="solver_cvg" localSheetId="35" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="36" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="37" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="41" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="32" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="34" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
@@ -118,6 +123,7 @@
     <definedName name="solver_drv" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_drv" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
@@ -132,6 +138,7 @@
     <definedName name="solver_eng" localSheetId="35" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="36" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="37" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="41" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_eng_1" localSheetId="4">2</definedName>
@@ -155,6 +162,7 @@
     <definedName name="solver_est" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_est_1" localSheetId="4">1</definedName>
@@ -178,6 +186,7 @@
     <definedName name="solver_itr" localSheetId="35" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="36" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="37" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="41" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_itr_1" localSheetId="4">2147483647</definedName>
@@ -201,6 +210,7 @@
     <definedName name="solver_lhs1" localSheetId="35" hidden="1">'Dual 2'!$E$10</definedName>
     <definedName name="solver_lhs1" localSheetId="36" hidden="1">'EJ3'!$E$10</definedName>
     <definedName name="solver_lhs1" localSheetId="37" hidden="1">EJ3_B!$E$10</definedName>
+    <definedName name="solver_lhs1" localSheetId="41" hidden="1">'EJ4'!$H$10</definedName>
     <definedName name="solver_lhs1" localSheetId="32" hidden="1">'Primal 1'!$E$10</definedName>
     <definedName name="solver_lhs1" localSheetId="34" hidden="1">'Primal 2'!$G$10</definedName>
     <definedName name="solver_lhs1_1" localSheetId="4">'2'!$D$7</definedName>
@@ -219,6 +229,7 @@
     <definedName name="solver_lhs2" localSheetId="35" hidden="1">'Dual 2'!$E$11</definedName>
     <definedName name="solver_lhs2" localSheetId="36" hidden="1">'EJ3'!$E$11</definedName>
     <definedName name="solver_lhs2" localSheetId="37" hidden="1">EJ3_B!$E$11</definedName>
+    <definedName name="solver_lhs2" localSheetId="41" hidden="1">'EJ4'!$H$11</definedName>
     <definedName name="solver_lhs2" localSheetId="32" hidden="1">'Primal 1'!$E$11</definedName>
     <definedName name="solver_lhs2" localSheetId="34" hidden="1">'Primal 2'!$G$8</definedName>
     <definedName name="solver_lhs2_1" localSheetId="4">'2'!$D$8</definedName>
@@ -235,6 +246,7 @@
     <definedName name="solver_lhs3" localSheetId="35" hidden="1">'Dual 2'!$E$12</definedName>
     <definedName name="solver_lhs3" localSheetId="36" hidden="1">'EJ3'!$E$7</definedName>
     <definedName name="solver_lhs3" localSheetId="37" hidden="1">EJ3_B!$E$7</definedName>
+    <definedName name="solver_lhs3" localSheetId="41" hidden="1">'EJ4'!$H$12</definedName>
     <definedName name="solver_lhs3" localSheetId="32" hidden="1">'Primal 1'!$E$8</definedName>
     <definedName name="solver_lhs3" localSheetId="34" hidden="1">'Primal 2'!$G$9</definedName>
     <definedName name="solver_lhs3_1" localSheetId="8">'3'!$H$9</definedName>
@@ -245,6 +257,7 @@
     <definedName name="solver_lhs4" localSheetId="35" hidden="1">'Dual 2'!$E$8</definedName>
     <definedName name="solver_lhs4" localSheetId="36" hidden="1">'EJ3'!$E$8</definedName>
     <definedName name="solver_lhs4" localSheetId="37" hidden="1">EJ3_B!$E$8</definedName>
+    <definedName name="solver_lhs4" localSheetId="41" hidden="1">'EJ4'!$H$8</definedName>
     <definedName name="solver_lhs4" localSheetId="32" hidden="1">'Primal 1'!$E$9</definedName>
     <definedName name="solver_lhs5" localSheetId="12" hidden="1">'4'!$F$10</definedName>
     <definedName name="solver_lhs5" localSheetId="24" hidden="1">'7'!$F$14</definedName>
@@ -252,6 +265,7 @@
     <definedName name="solver_lhs5" localSheetId="35" hidden="1">'Dual 2'!$E$9</definedName>
     <definedName name="solver_lhs5" localSheetId="36" hidden="1">'EJ3'!$E$9</definedName>
     <definedName name="solver_lhs5" localSheetId="37" hidden="1">EJ3_B!$E$9</definedName>
+    <definedName name="solver_lhs5" localSheetId="41" hidden="1">'EJ4'!$H$9</definedName>
     <definedName name="solver_lhs6" localSheetId="12" hidden="1">'4'!$F$9</definedName>
     <definedName name="solver_lhs6" localSheetId="24" hidden="1">'7'!$F$15</definedName>
     <definedName name="solver_lhs6" localSheetId="28" hidden="1">'8'!$E$9</definedName>
@@ -279,6 +293,7 @@
     <definedName name="solver_mip" localSheetId="35" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="36" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="37" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="41" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
@@ -293,6 +308,7 @@
     <definedName name="solver_mni" localSheetId="35" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="36" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="37" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="41" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="32" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="34" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
@@ -307,6 +323,7 @@
     <definedName name="solver_mrt" localSheetId="35" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="36" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="37" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="41" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="32" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="34" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
@@ -321,6 +338,7 @@
     <definedName name="solver_msl" localSheetId="35" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="36" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="37" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="41" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_mtpb" localSheetId="16">0</definedName>
@@ -338,6 +356,7 @@
     <definedName name="solver_neg" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_neg_1" localSheetId="4">1</definedName>
@@ -355,6 +374,7 @@
     <definedName name="solver_nod" localSheetId="35" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="36" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="37" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="41" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
@@ -369,6 +389,7 @@
     <definedName name="solver_num" localSheetId="35" hidden="1">5</definedName>
     <definedName name="solver_num" localSheetId="36" hidden="1">5</definedName>
     <definedName name="solver_num" localSheetId="37" hidden="1">5</definedName>
+    <definedName name="solver_num" localSheetId="41" hidden="1">5</definedName>
     <definedName name="solver_num" localSheetId="32" hidden="1">4</definedName>
     <definedName name="solver_num" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_num_1" localSheetId="4">3</definedName>
@@ -386,6 +407,7 @@
     <definedName name="solver_nwt" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_nwt_1" localSheetId="4">1</definedName>
@@ -403,6 +425,7 @@
     <definedName name="solver_opt" localSheetId="35" hidden="1">'Dual 2'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="36" hidden="1">'EJ3'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="37" hidden="1">EJ3_B!$B$1</definedName>
+    <definedName name="solver_opt" localSheetId="41" hidden="1">'EJ4'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="32" hidden="1">'Primal 1'!$B$1</definedName>
     <definedName name="solver_opt" localSheetId="34" hidden="1">'Primal 2'!$B$1</definedName>
     <definedName name="solver_opt_1" localSheetId="4">'2'!$B$1</definedName>
@@ -420,6 +443,7 @@
     <definedName name="solver_pre" localSheetId="35" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="36" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="37" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="41" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="32" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="34" hidden="1">0.000001</definedName>
     <definedName name="solver_pre_1" localSheetId="4">0</definedName>
@@ -440,6 +464,7 @@
     <definedName name="solver_rbv" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_rbv" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
@@ -454,6 +479,7 @@
     <definedName name="solver_rel1" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="41" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_rel1_1" localSheetId="4">1</definedName>
@@ -472,6 +498,7 @@
     <definedName name="solver_rel2" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="41" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel2" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_rel2_1" localSheetId="4">1</definedName>
@@ -488,6 +515,7 @@
     <definedName name="solver_rel3" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_rel3" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="41" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_rel3_1" localSheetId="8">3</definedName>
@@ -498,6 +526,7 @@
     <definedName name="solver_rel4" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_rel5" localSheetId="12" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="24" hidden="1">3</definedName>
@@ -505,6 +534,7 @@
     <definedName name="solver_rel5" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="12" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="24" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="28" hidden="1">1</definedName>
@@ -524,6 +554,7 @@
     <definedName name="solver_rhs1" localSheetId="35" hidden="1">'Dual 2'!$G$10</definedName>
     <definedName name="solver_rhs1" localSheetId="36" hidden="1">'EJ3'!$G$10</definedName>
     <definedName name="solver_rhs1" localSheetId="37" hidden="1">EJ3_B!$G$10</definedName>
+    <definedName name="solver_rhs1" localSheetId="41" hidden="1">'EJ4'!$J$10</definedName>
     <definedName name="solver_rhs1" localSheetId="32" hidden="1">'Primal 1'!$G$10</definedName>
     <definedName name="solver_rhs1" localSheetId="34" hidden="1">'Primal 2'!$I$10</definedName>
     <definedName name="solver_rhs1_1" localSheetId="4">'2'!$F$7</definedName>
@@ -542,6 +573,7 @@
     <definedName name="solver_rhs2" localSheetId="35" hidden="1">'Dual 2'!$G$11</definedName>
     <definedName name="solver_rhs2" localSheetId="36" hidden="1">'EJ3'!$G$11</definedName>
     <definedName name="solver_rhs2" localSheetId="37" hidden="1">EJ3_B!$G$11</definedName>
+    <definedName name="solver_rhs2" localSheetId="41" hidden="1">'EJ4'!$J$11</definedName>
     <definedName name="solver_rhs2" localSheetId="32" hidden="1">'Primal 1'!$G$11</definedName>
     <definedName name="solver_rhs2" localSheetId="34" hidden="1">'Primal 2'!$I$8</definedName>
     <definedName name="solver_rhs2_1" localSheetId="4">'2'!$F$8</definedName>
@@ -558,6 +590,7 @@
     <definedName name="solver_rhs3" localSheetId="35" hidden="1">'Dual 2'!$G$12</definedName>
     <definedName name="solver_rhs3" localSheetId="36" hidden="1">'EJ3'!$G$7</definedName>
     <definedName name="solver_rhs3" localSheetId="37" hidden="1">EJ3_B!$G$7</definedName>
+    <definedName name="solver_rhs3" localSheetId="41" hidden="1">'EJ4'!$J$12</definedName>
     <definedName name="solver_rhs3" localSheetId="32" hidden="1">'Primal 1'!$G$8</definedName>
     <definedName name="solver_rhs3" localSheetId="34" hidden="1">'Primal 2'!$I$9</definedName>
     <definedName name="solver_rhs3_1" localSheetId="8">'3'!$J$9</definedName>
@@ -568,6 +601,7 @@
     <definedName name="solver_rhs4" localSheetId="35" hidden="1">'Dual 2'!$G$8</definedName>
     <definedName name="solver_rhs4" localSheetId="36" hidden="1">'EJ3'!$G$8</definedName>
     <definedName name="solver_rhs4" localSheetId="37" hidden="1">EJ3_B!$G$8</definedName>
+    <definedName name="solver_rhs4" localSheetId="41" hidden="1">'EJ4'!$J$8</definedName>
     <definedName name="solver_rhs4" localSheetId="32" hidden="1">'Primal 1'!$G$9</definedName>
     <definedName name="solver_rhs5" localSheetId="12" hidden="1">'4'!$H$10</definedName>
     <definedName name="solver_rhs5" localSheetId="24" hidden="1">'7'!$H$14</definedName>
@@ -575,6 +609,7 @@
     <definedName name="solver_rhs5" localSheetId="35" hidden="1">'Dual 2'!$G$9</definedName>
     <definedName name="solver_rhs5" localSheetId="36" hidden="1">'EJ3'!$G$9</definedName>
     <definedName name="solver_rhs5" localSheetId="37" hidden="1">EJ3_B!$G$9</definedName>
+    <definedName name="solver_rhs5" localSheetId="41" hidden="1">'EJ4'!$J$9</definedName>
     <definedName name="solver_rhs6" localSheetId="12" hidden="1">'4'!$H$9</definedName>
     <definedName name="solver_rhs6" localSheetId="24" hidden="1">'7'!$H$15</definedName>
     <definedName name="solver_rhs6" localSheetId="28" hidden="1">'8'!$G$9</definedName>
@@ -594,6 +629,7 @@
     <definedName name="solver_rlx" localSheetId="35" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="36" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="37" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="41" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
@@ -608,6 +644,7 @@
     <definedName name="solver_rsd" localSheetId="35" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="36" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="37" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="41" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="32" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="34" hidden="1">0</definedName>
     <definedName name="solver_rsp" localSheetId="16">0</definedName>
@@ -625,6 +662,7 @@
     <definedName name="solver_scl" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_scl" localSheetId="41" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="32" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="34" hidden="1">1</definedName>
     <definedName name="solver_scl_1" localSheetId="4">1</definedName>
@@ -642,7 +680,9 @@
     <definedName name="solver_sho" localSheetId="35" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="36" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="37" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="41" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="44" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="5" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="9" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="13" hidden="1">2</definedName>
@@ -677,6 +717,7 @@
     <definedName name="solver_ssz" localSheetId="35" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="36" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="37" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="41" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="32" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="34" hidden="1">100</definedName>
     <definedName name="solver_stol" localSheetId="16">0.000001</definedName>
@@ -694,6 +735,7 @@
     <definedName name="solver_tim" localSheetId="35" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="36" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="37" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="41" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="32" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="34" hidden="1">2147483647</definedName>
     <definedName name="solver_tim_1" localSheetId="4">2147483647</definedName>
@@ -711,6 +753,7 @@
     <definedName name="solver_tol" localSheetId="35" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="36" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="37" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="41" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="32" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="34" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
@@ -725,6 +768,7 @@
     <definedName name="solver_typ" localSheetId="35" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="36" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="37" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="41" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="32" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="34" hidden="1">2</definedName>
     <definedName name="solver_typ_1" localSheetId="4">1</definedName>
@@ -742,6 +786,7 @@
     <definedName name="solver_val" localSheetId="35" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="36" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="37" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="41" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="32" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="34" hidden="1">0</definedName>
     <definedName name="solver_val_1" localSheetId="4">0</definedName>
@@ -759,6 +804,7 @@
     <definedName name="solver_ver" localSheetId="35" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="36" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="37" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="41" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="32" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="34" hidden="1">3</definedName>
     <definedName name="solver_ver_1" localSheetId="4">3</definedName>
@@ -787,7 +833,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="310">
   <si>
     <t>Objetivo</t>
   </si>
@@ -1660,6 +1706,63 @@
   </si>
   <si>
     <t>Informe creado: 23/4/2026 11:08:58</t>
+  </si>
+  <si>
+    <t>X11</t>
+  </si>
+  <si>
+    <t>X12</t>
+  </si>
+  <si>
+    <t>X13</t>
+  </si>
+  <si>
+    <t>X21</t>
+  </si>
+  <si>
+    <t>X22</t>
+  </si>
+  <si>
+    <t>X23</t>
+  </si>
+  <si>
+    <t>Hoja de cálculo: [TP3.xlsx]EJ4</t>
+  </si>
+  <si>
+    <t>Informe creado: 23/4/2026 11:31:09</t>
+  </si>
+  <si>
+    <t>Tiempo de la solución: 0,031 segundos.</t>
+  </si>
+  <si>
+    <t>$F$4</t>
+  </si>
+  <si>
+    <t>$G$4</t>
+  </si>
+  <si>
+    <t>$H$10</t>
+  </si>
+  <si>
+    <t>$H$10&gt;=$J$10</t>
+  </si>
+  <si>
+    <t>$H$11</t>
+  </si>
+  <si>
+    <t>$H$11&gt;=$J$11</t>
+  </si>
+  <si>
+    <t>$H$12</t>
+  </si>
+  <si>
+    <t>$H$12&gt;=$J$12</t>
+  </si>
+  <si>
+    <t>$H$8&lt;=$J$8</t>
+  </si>
+  <si>
+    <t>$H$9&lt;=$J$9</t>
   </si>
 </sst>
 </file>
@@ -11926,9 +12029,1144 @@
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1E2C01-65FB-4999-9D74-801357ABBFE6}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="6.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="4.875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B1">
+        <f>SUMPRODUCT(B4:G4,B5:G5)</f>
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C3" t="s">
+        <v>292</v>
+      </c>
+      <c r="D3" t="s">
+        <v>293</v>
+      </c>
+      <c r="E3" t="s">
+        <v>294</v>
+      </c>
+      <c r="F3" t="s">
+        <v>295</v>
+      </c>
+      <c r="G3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>6000</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>4000</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>8000</v>
+      </c>
+      <c r="G4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>8</v>
+      </c>
+      <c r="F5">
+        <v>7</v>
+      </c>
+      <c r="G5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <f>SUMPRODUCT(B4:G4,B8:G8)</f>
+        <v>10000</v>
+      </c>
+      <c r="I8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <f>SUMPRODUCT(B4:G4,B9:G9)</f>
+        <v>9000</v>
+      </c>
+      <c r="I9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <f>SUMPRODUCT(B4:G4,B10:G10)</f>
+        <v>6000</v>
+      </c>
+      <c r="I10" t="s">
+        <v>73</v>
+      </c>
+      <c r="J10">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <f>SUMPRODUCT(B4:G4,B11:G11)</f>
+        <v>8000</v>
+      </c>
+      <c r="I11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J11">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <f>SUMPRODUCT(B4:G4,B12:G12)</f>
+        <v>5000</v>
+      </c>
+      <c r="I12" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12">
+        <v>5000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B638F2D-101B-4A5B-A9BB-2CD72E40C1E0}">
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.125" customWidth="1"/>
+    <col min="2" max="2" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="14">
+        <v>0</v>
+      </c>
+      <c r="E16" s="14">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="D21" s="15">
+        <v>0</v>
+      </c>
+      <c r="E21" s="15">
+        <v>6000</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B22" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="D22" s="15">
+        <v>0</v>
+      </c>
+      <c r="E22" s="15">
+        <v>0</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B23" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="D23" s="15">
+        <v>0</v>
+      </c>
+      <c r="E23" s="15">
+        <v>4000</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D24" s="15">
+        <v>0</v>
+      </c>
+      <c r="E24" s="15">
+        <v>0</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B25" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="D25" s="15">
+        <v>0</v>
+      </c>
+      <c r="E25" s="15">
+        <v>8000</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="D26" s="14">
+        <v>0</v>
+      </c>
+      <c r="E26" s="14">
+        <v>1000</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="13" t="s">
+        <v>302</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="15">
+        <v>6000</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G31" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B32" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="C32" s="13"/>
+      <c r="D32" s="15">
+        <v>8000</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G32" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B33" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="15">
+        <v>5000</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G33" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B34" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" s="13"/>
+      <c r="D34" s="15">
+        <v>10000</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G34" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="D35" s="14">
+        <v>9000</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="G35" s="11">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B934FF51-80CB-46E4-891E-344D2E471D43}">
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.125" customWidth="1"/>
+    <col min="2" max="2" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B9" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="D9" s="13">
+        <v>6000</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <v>5</v>
+      </c>
+      <c r="G9" s="13">
+        <v>1</v>
+      </c>
+      <c r="H9" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B10" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13">
+        <v>6</v>
+      </c>
+      <c r="G10" s="13">
+        <v>1E+30</v>
+      </c>
+      <c r="H10" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B11" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="D11" s="13">
+        <v>4000</v>
+      </c>
+      <c r="E11" s="13">
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
+        <v>8</v>
+      </c>
+      <c r="G11" s="13">
+        <v>1</v>
+      </c>
+      <c r="H11" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B12" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D12" s="13">
+        <v>0</v>
+      </c>
+      <c r="E12" s="13">
+        <v>1</v>
+      </c>
+      <c r="F12" s="13">
+        <v>8</v>
+      </c>
+      <c r="G12" s="13">
+        <v>1E+30</v>
+      </c>
+      <c r="H12" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B13" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="D13" s="13">
+        <v>8000</v>
+      </c>
+      <c r="E13" s="13">
+        <v>0</v>
+      </c>
+      <c r="F13" s="13">
+        <v>7</v>
+      </c>
+      <c r="G13" s="13">
+        <v>1</v>
+      </c>
+      <c r="H13" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="D14" s="11">
+        <v>1000</v>
+      </c>
+      <c r="E14" s="11">
+        <v>0</v>
+      </c>
+      <c r="F14" s="11">
+        <v>10</v>
+      </c>
+      <c r="G14" s="11">
+        <v>1</v>
+      </c>
+      <c r="H14" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="H18" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B19" s="13" t="s">
+        <v>302</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13">
+        <v>6000</v>
+      </c>
+      <c r="E19" s="13">
+        <v>7</v>
+      </c>
+      <c r="F19" s="13">
+        <v>6000</v>
+      </c>
+      <c r="G19" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H19" s="13">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13">
+        <v>8000</v>
+      </c>
+      <c r="E20" s="13">
+        <v>7</v>
+      </c>
+      <c r="F20" s="13">
+        <v>8000</v>
+      </c>
+      <c r="G20" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H20" s="13">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B21" s="13" t="s">
+        <v>306</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13">
+        <v>5000</v>
+      </c>
+      <c r="E21" s="13">
+        <v>10</v>
+      </c>
+      <c r="F21" s="13">
+        <v>5000</v>
+      </c>
+      <c r="G21" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H21" s="13">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B22" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13">
+        <v>10000</v>
+      </c>
+      <c r="E22" s="13">
+        <v>-2</v>
+      </c>
+      <c r="F22" s="13">
+        <v>10000</v>
+      </c>
+      <c r="G22" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H22" s="13">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11">
+        <v>9000</v>
+      </c>
+      <c r="E23" s="11">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11">
+        <v>10000</v>
+      </c>
+      <c r="G23" s="11">
+        <v>1E+30</v>
+      </c>
+      <c r="H23" s="11">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF2099D4-F57C-467D-BB72-7FE0943E3EA1}">
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.125" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.125" customWidth="1"/>
+    <col min="6" max="6" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="2.125" customWidth="1"/>
+    <col min="9" max="9" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="B6" s="16"/>
+      <c r="C6" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="14">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="B11" s="16"/>
+      <c r="C11" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="F11" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="I11" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="J11" s="16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B13" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="D13" s="15">
+        <v>6000</v>
+      </c>
+      <c r="F13" s="15">
+        <v>6000</v>
+      </c>
+      <c r="G13" s="15">
+        <v>128000</v>
+      </c>
+      <c r="I13" s="15">
+        <v>6000</v>
+      </c>
+      <c r="J13" s="15">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="D14" s="15">
+        <v>0</v>
+      </c>
+      <c r="F14" s="15">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15">
+        <v>128000</v>
+      </c>
+      <c r="I14" s="15">
+        <v>0</v>
+      </c>
+      <c r="J14" s="15">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B15" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="D15" s="15">
+        <v>4000</v>
+      </c>
+      <c r="F15" s="15">
+        <v>4000</v>
+      </c>
+      <c r="G15" s="15">
+        <v>128000</v>
+      </c>
+      <c r="I15" s="15">
+        <v>4000</v>
+      </c>
+      <c r="J15" s="15">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B16" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D16" s="15">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15">
+        <v>128000</v>
+      </c>
+      <c r="I16" s="15">
+        <v>1000</v>
+      </c>
+      <c r="J16" s="15">
+        <v>136000</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B17" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="D17" s="15">
+        <v>8000</v>
+      </c>
+      <c r="F17" s="15">
+        <v>8000</v>
+      </c>
+      <c r="G17" s="15">
+        <v>128000</v>
+      </c>
+      <c r="I17" s="15">
+        <v>9000</v>
+      </c>
+      <c r="J17" s="15">
+        <v>135000</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="D18" s="14">
+        <v>1000</v>
+      </c>
+      <c r="F18" s="14">
+        <v>1000</v>
+      </c>
+      <c r="G18" s="14">
+        <v>128000</v>
+      </c>
+      <c r="I18" s="14">
+        <v>2000</v>
+      </c>
+      <c r="J18" s="14">
+        <v>138000</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>